<commit_message>
added new sheet in excel
</commit_message>
<xml_diff>
--- a/data/tips.xlsx
+++ b/data/tips.xlsx
@@ -7,13 +7,16 @@
     <sheet name="list" sheetId="2" r:id="rId2"/>
     <sheet name="stack&amp;deque" sheetId="3" r:id="rId3"/>
     <sheet name="string" sheetId="4" r:id="rId4"/>
-    <sheet name="char" sheetId="5" r:id="rId5"/>
-    <sheet name="int" sheetId="6" r:id="rId6"/>
-    <sheet name="Sheet2" sheetId="7" r:id="rId7"/>
-    <sheet name="hashset" sheetId="8" r:id="rId8"/>
-    <sheet name="hashmap" sheetId="9" r:id="rId9"/>
-    <sheet name="PriorityQueue" sheetId="10" r:id="rId10"/>
-    <sheet name="stream" sheetId="11" r:id="rId11"/>
+    <sheet name="Sheet3" sheetId="5" r:id="rId5"/>
+    <sheet name="char" sheetId="6" r:id="rId6"/>
+    <sheet name="int" sheetId="7" r:id="rId7"/>
+    <sheet name="Sheet2" sheetId="8" r:id="rId8"/>
+    <sheet name="hashset" sheetId="9" r:id="rId9"/>
+    <sheet name="hashmap" sheetId="10" r:id="rId10"/>
+    <sheet name="PriorityQueue" sheetId="11" r:id="rId11"/>
+    <sheet name="stream" sheetId="12" r:id="rId12"/>
+    <sheet name="数组集合互换" sheetId="13" r:id="rId13"/>
+    <sheet name="Sheet5" sheetId="14" r:id="rId14"/>
   </sheets>
 </workbook>
 </file>
@@ -407,7 +410,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D29"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -423,15 +426,12 @@
         <v>例子</v>
       </c>
     </row>
-    <row r="2" xml:space="preserve">
-      <c r="A2" t="str" xml:space="preserve">
-        <v xml:space="preserve">Arrays.sort(arr)
-Arrays.sort(words, (a, b) -&gt; {
-            return a.charAt(a.length() - 1) - b.charAt(b.length() - 1);
-        });</v>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Arrays.sort(arr)</v>
       </c>
       <c r="B2" t="str">
-        <v>排序，或 指定的元素在数组里比较</v>
+        <v>排序</v>
       </c>
       <c r="C2" t="str">
         <v>升序排序只好升序，降序要另外实现</v>
@@ -448,8 +448,8 @@
         <v>数组必须是对象 Integer[]，不能是 int[]</v>
       </c>
       <c r="D3" t="str" xml:space="preserve">
-        <v xml:space="preserve">Integer[] arr = {5, 2, 8, 1, 3};
-Arrays.sort(arr, Collections.reverseOrder());
+        <v xml:space="preserve">Integer[] arr = {5, 2, 8, 1, 3};_x000d_
+Arrays.sort(arr, Collections.reverseOrder());_x000d_
 System.out.println(Arrays.toString(arr));</v>
       </c>
     </row>
@@ -458,14 +458,14 @@
         <v>Arrays.binarySearch(arr, key)</v>
       </c>
       <c r="B4" t="str" xml:space="preserve">
-        <v xml:space="preserve">二分查找，返回索引，
+        <v xml:space="preserve">二分查找，返回索引，_x000d_
 用来在 已排序数组 中快速查找元素的位置</v>
       </c>
       <c r="C4" t="str">
         <v>-1 表示未找到</v>
       </c>
       <c r="D4" t="str" xml:space="preserve">
-        <v xml:space="preserve">int index = Arrays.binarySearch(array, key);
+        <v xml:space="preserve">int index = Arrays.binarySearch(array, key);_x000d_
 int idx = Arrays.binarySearch(nums, 1, 4, 3);//	fromIndex = 1 (包含)，toIndex = 4 (不包含)，在子区间 [1,4) 查找 3</v>
       </c>
     </row>
@@ -491,7 +491,7 @@
         <v>把数组的所有元素填充为同一个值</v>
       </c>
       <c r="D6" t="str" xml:space="preserve">
-        <v xml:space="preserve">int[] arr = new int[5];
+        <v xml:space="preserve">int[] arr = new int[5];_x000d_
 Arrays.fill(arr, 3);// [3, 3, 3, 3, 3]</v>
       </c>
     </row>
@@ -500,14 +500,14 @@
         <v>Arrays.copyOf(arr, len)</v>
       </c>
       <c r="B7" t="str" xml:space="preserve">
-        <v xml:space="preserve">复制一个数组，生成指定长度的新数组，
+        <v xml:space="preserve">复制一个数组，生成指定长度的新数组，_x000d_
 可以动态改变数组的长度，和clone()的区别</v>
       </c>
       <c r="C7" t="str">
         <v>指定长度</v>
       </c>
       <c r="D7" t="str" xml:space="preserve">
-        <v xml:space="preserve">int[] arr = {1, 2, 3, 4};
+        <v xml:space="preserve">int[] arr = {1, 2, 3, 4};_x000d_
 int[] newArr = Arrays.copyOf(arr, 3);</v>
       </c>
     </row>
@@ -516,14 +516,14 @@
         <v>Arrays.copyOfRange(arr, from, to)</v>
       </c>
       <c r="B8" t="str" xml:space="preserve">
-        <v xml:space="preserve">截取子数组，复制部分数组，
+        <v xml:space="preserve">截取子数组，复制部分数组，_x000d_
 新成新数组，左闭右开</v>
       </c>
       <c r="C8" t="str">
         <v>复制 index 从 from 到 to-1 的元素</v>
       </c>
       <c r="D8" t="str" xml:space="preserve">
-        <v xml:space="preserve">int[] arr = {10,20,30,40,50};
+        <v xml:space="preserve">int[] arr = {10,20,30,40,50};_x000d_
 int[] newArr = Arrays.copyOfRange(arr, 1, 4);//[20, 30, 40]</v>
       </c>
     </row>
@@ -532,16 +532,16 @@
         <v>System.arraycopy 高性能复制</v>
       </c>
       <c r="B9" t="str" xml:space="preserve">
-        <v xml:space="preserve">arraycopy(src,0,dst,0,n)
+        <v xml:space="preserve">arraycopy(src,0,dst,0,n)_x000d_
 //源头，源头起始位置，目标新数组，目标数组起始位置，复制长度</v>
       </c>
       <c r="C9" t="str">
         <v/>
       </c>
       <c r="D9" t="str" xml:space="preserve">
-        <v xml:space="preserve">int[] nums = {1,2,3,4,5};
-int[] copy = new int[5];
-System.arraycopy(nums, 0, copy, 0, nums.length);
+        <v xml:space="preserve">int[] nums = {1,2,3,4,5};_x000d_
+int[] copy = new int[5];_x000d_
+System.arraycopy(nums, 0, copy, 0, nums.length);_x000d_
 System.out.println(Arrays.toString(copy));//[1, 2, 3, 4, 5]</v>
       </c>
     </row>
@@ -572,29 +572,29 @@
         <v>Arrays.stream(arr)</v>
       </c>
       <c r="B12" t="str" xml:space="preserve">
-        <v xml:space="preserve">把数组转换成 IntStream（流）对象，
-然后可以用 函数式操作（lambada）处理数据，比如 sum()、max(), average(),distinct(), filter()、map() 等。
+        <v xml:space="preserve">把数组转换成 IntStream（流）对象，_x000d_
+然后可以用 函数式操作（lambada）处理数据，比如 sum()、max(), average(),distinct(), filter()、map() 等。_x000d_
 .stream() 不一定是 IntStream，要看来源类型。如果来源是对象List&lt;Integer&gt; list = List.of(1,2,3); list.stream()得到是Stream&lt;Integer&gt;。同理Integer[] arr = {1,2,3};Arrays.stream(arr);但是，int[] nums = {1,2,3};Arrays.stream(nums)，得到是Intstream可以用那些方法。用mapToInt为了能用到max() 这样的函数方法。</v>
       </c>
       <c r="C12" t="str" xml:space="preserve">
-        <v xml:space="preserve">Arrays.stream(arr)//返回IntStream对象
-int[] arr = {1,2,3,4};int sum = Arrays.stream(arr).sum();
+        <v xml:space="preserve">Arrays.stream(arr)//返回IntStream对象_x000d_
+int[] arr = {1,2,3,4};int sum = Arrays.stream(arr).sum();_x000d_
 求最大值：int max = Arrays.stream(arr).max()/.min().getAsInt();</v>
       </c>
       <c r="D12" t="str" xml:space="preserve">
-        <v xml:space="preserve">过滤数据：int[] arr = {1,2,3,4,5,6};
-Arrays.stream(arr) .filter(n -&gt; n % 2 == 0).forEach(System.out::println);
-map转换：
-int[] arr = {1,2,3};
-Arrays.stream(arr).map(n -&gt; n * 2).forEach(System.out::println);//246
-数组转list：
-int[] arr = {1,2,3}
-List&lt;Integer&gt; list =Arrays.stream(arr).boxed().toList();
-boxed()为了装箱成Stream对象Stream&lt;Integer&gt;，Stream是用来操作数据集合的。
-计数：
-int[] arr = {1,2,3,4,5};
-long count =Arrays.stream(arr).filter(n -&gt; n &gt; 3).count(); // 4，5
-去重并建立新数组：
+        <v xml:space="preserve">过滤数据：int[] arr = {1,2,3,4,5,6};_x000d_
+Arrays.stream(arr) .filter(n -&gt; n % 2 == 0).forEach(System.out::println);_x000d_
+map转换：_x000d_
+int[] arr = {1,2,3};_x000d_
+Arrays.stream(arr).map(n -&gt; n * 2).forEach(System.out::println);//246_x000d_
+数组转list：_x000d_
+int[] arr = {1,2,3}_x000d_
+List&lt;Integer&gt; list =Arrays.stream(arr).boxed().toList();_x000d_
+boxed()为了装箱成Stream对象Stream&lt;Integer&gt;，Stream是用来操作数据集合的。_x000d_
+计数：_x000d_
+int[] arr = {1,2,3,4,5};_x000d_
+long count =Arrays.stream(arr).filter(n -&gt; n &gt; 3).count(); // 4，5_x000d_
+去重并建立新数组：_x000d_
 int[] newArr = Arrays.stream(nums).distinct().toArray();</v>
       </c>
     </row>
@@ -609,8 +609,8 @@
         <v>List 只能存对象</v>
       </c>
       <c r="D13" t="str" xml:space="preserve">
-        <v xml:space="preserve">int[] nums = {1,2,3,4};
-List&lt;Integer&gt; list =Arrays.stream(nums).boxed().toList();
+        <v xml:space="preserve">int[] nums = {1,2,3,4};_x000d_
+List&lt;Integer&gt; list =Arrays.stream(nums).boxed().toList();_x000d_
 System.out.println(list);</v>
       </c>
     </row>
@@ -625,8 +625,8 @@
         <v>Arrays.asList(array)，Arrays.asList() 返回的是固定大小的数组，底层仍是array，不可以list.add，remove,可以修改元素。</v>
       </c>
       <c r="D14" t="str" xml:space="preserve">
-        <v xml:space="preserve">String[] arr = {"apple", "banana", "cat"};
-List&lt;String&gt; list = Arrays.asList(arr);
+        <v xml:space="preserve">String[] arr = {"apple", "banana", "cat"};_x000d_
+List&lt;String&gt; list = Arrays.asList(arr);_x000d_
 System.out.println(list);</v>
       </c>
     </row>
@@ -635,20 +635,20 @@
         <v>如果想要真正的 ArrayList</v>
       </c>
       <c r="B15" t="str" xml:space="preserve">
-        <v xml:space="preserve">List&lt;Integer&gt; list =
+        <v xml:space="preserve">List&lt;Integer&gt; list =_x000d_
     new ArrayList&lt;&gt;(Arrays.asList(1,2,3));</v>
       </c>
     </row>
     <row r="16" xml:space="preserve">
       <c r="A16" t="str" xml:space="preserve">
-        <v xml:space="preserve">list.toArray(new Integer[0]);
+        <v xml:space="preserve">list.toArray(new Integer[0]);_x000d_
 List-&gt;数组</v>
       </c>
       <c r="B16" t="str">
         <v/>
       </c>
       <c r="C16" t="str" xml:space="preserve">
-        <v xml:space="preserve">list.toArray(new Integer[0])返回类型是
+        <v xml:space="preserve">list.toArray(new Integer[0])返回类型是_x000d_
 Integer[]， Java 会自动创建正确大小数组。等价于list.toArray(new Integer[list.size()])。list.toArray()返回类型是Object[]</v>
       </c>
       <c r="D16" t="str">
@@ -671,11 +671,11 @@
         <v>int[] newArr = oldarr.clone()</v>
       </c>
       <c r="C18" t="str" xml:space="preserve">
-        <v xml:space="preserve">创建一个内容一样的新副本（浅拷贝）,clone 后修改 新数组copy 不影响 nums。Arrays.copyOf()
+        <v xml:space="preserve">创建一个内容一样的新副本（浅拷贝）,clone 后修改 新数组copy 不影响 nums。Arrays.copyOf()_x000d_
 可以改变长度</v>
       </c>
       <c r="D18" t="str" xml:space="preserve">
-        <v xml:space="preserve">int[] nums = {1,2,3};
+        <v xml:space="preserve">int[] nums = {1,2,3};_x000d_
 int[] copy = nums.clone();</v>
       </c>
     </row>
@@ -765,7 +765,7 @@
         <v>要降序（需要用 Integer[]）</v>
       </c>
       <c r="D25" t="str" xml:space="preserve">
-        <v xml:space="preserve">Integer[] nums = {5,2,8,1};
+        <v xml:space="preserve">Integer[] nums = {5,2,8,1};_x000d_
 Arrays.sort(nums, (a,b) -&gt; b - a);</v>
       </c>
     </row>
@@ -780,7 +780,7 @@
         <v/>
       </c>
       <c r="D26" t="str" xml:space="preserve">
-        <v xml:space="preserve">List&lt;Integer&gt; list = Arrays.asList(5,2,8,1);
+        <v xml:space="preserve">List&lt;Integer&gt; list = Arrays.asList(5,2,8,1);_x000d_
 list.sort((a,b) -&gt; a - b);// 升序</v>
       </c>
     </row>
@@ -795,9 +795,9 @@
         <v/>
       </c>
       <c r="D27" t="str" xml:space="preserve">
-        <v xml:space="preserve">Arrays.sort(arr, Comparator.comparingInt(a -&gt; a[1]));// 升序
-Arrays.sort(arr,
-    Comparator.comparingInt((int[] a) -&gt; a[1]).reversed()
+        <v xml:space="preserve">Arrays.sort(arr, Comparator.comparingInt(a -&gt; a[1]));// 升序_x000d_
+Arrays.sort(arr,_x000d_
+    Comparator.comparingInt((int[] a) -&gt; a[1]).reversed()_x000d_
 );//降序</v>
       </c>
     </row>
@@ -823,48 +823,997 @@
         <v/>
       </c>
       <c r="D29" t="str" xml:space="preserve">
-        <v xml:space="preserve">int[] a = {1,2,3};
-int[] b = {1,2,3};
-int[] c = {3,2,1};
+        <v xml:space="preserve">int[] a = {1,2,3};_x000d_
+int[] b = {1,2,3};_x000d_
+int[] c = {3,2,1};_x000d_
+_x000d_
 System.out.println(Arrays.equals(a, b)); // true</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D29"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D20"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>方法</v>
+      </c>
+      <c r="B1" t="str">
+        <v>功能</v>
+      </c>
+      <c r="C1" t="str">
+        <v>备注</v>
+      </c>
+      <c r="D1" t="str">
+        <v>例子</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Map&lt;String, Integer&gt; map = new HashMap&lt;&gt;();</v>
+      </c>
+      <c r="B2" t="str">
+        <v>创建一个空 HashMap</v>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3" t="str" xml:space="preserve">
+        <v xml:space="preserve">map.put("apple", 3); // 添加 key=apple, value=3_x000d_
+map.put("banana", 5); // 添加_x000d_
+map.put("apple", 10); // 更新 key=apple 的值为10</v>
+      </c>
+      <c r="B3" t="str">
+        <v>添加 / 更新元素</v>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str">
+        <v>map.put(key, map.getOrDefault(key, 0) + 1);</v>
+      </c>
+      <c r="B4" t="str">
+        <v>统计频率</v>
+      </c>
+      <c r="C4" t="str" xml:space="preserve">
+        <v xml:space="preserve">如果 key 已存在 → value +1_x000d_
+如果 key 不存在 → 默认 0 +1 → 放入 1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>map.getOrDefault("orange", 0);</v>
+      </c>
+      <c r="B5" t="str">
+        <v>统计出现次数，获取元素</v>
+      </c>
+      <c r="C5" t="str">
+        <v>int val2 = map.getOrDefault("orange", 0); // 不存在返回0</v>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6" t="str" xml:space="preserve">
+        <v xml:space="preserve">map.containsKey("apple"); // true_x000d_
+map.containsValue(10);    // true</v>
+      </c>
+      <c r="B6" t="str">
+        <v>判断 key / value</v>
+      </c>
+      <c r="C6" t="str" xml:space="preserve">
+        <v xml:space="preserve">map.containsKey("apple"); // true_x000d_
+map.containsValue(10);    // true</v>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
+      <c r="A7" t="str" xml:space="preserve">
+        <v xml:space="preserve">map.remove("banana");       // 删除 key=banana_x000d_
+map.remove("apple", 10);    // 删除 key=apple 且 value=10 的条目</v>
+      </c>
+      <c r="B7" t="str">
+        <v>删除元素</v>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
+      <c r="A8" t="str" xml:space="preserve">
+        <v xml:space="preserve">for (String key : map.keySet()) {_x000d_
+    System.out.println(key + " -&gt; " + map.get(key));_x000d_
+}</v>
+      </c>
+      <c r="B8" t="str">
+        <v>遍历 key</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>for (Integer value : map.values()) {System.out.println(value);}</v>
+      </c>
+      <c r="B9" t="str">
+        <v>遍历value</v>
+      </c>
+    </row>
+    <row r="10" xml:space="preserve">
+      <c r="A10" t="str" xml:space="preserve">
+        <v xml:space="preserve">for (Map.Entry&lt;String, Integer&gt; entry : map.entrySet()) {_x000d_
+    System.out.println(entry.getKey() + " -&gt; " + entry.getValue());_x000d_
+}</v>
+      </c>
+      <c r="B10" t="str">
+        <v>遍历Entry</v>
+      </c>
+    </row>
+    <row r="11" xml:space="preserve">
+      <c r="A11" t="str" xml:space="preserve">
+        <v xml:space="preserve">map.computeIfAbsent(key, k -&gt; value);_x000d_
+如果没有 key，就创建新的 ArrayList_x000d_
+            indexMap.computeIfAbsent(c, k -&gt; new ArrayList&lt;&gt;()).add(i);</v>
+      </c>
+      <c r="B11" t="str" xml:space="preserve">
+        <v xml:space="preserve">分组：computeIfAbsent_x000d_
+map.computeIfAbsent("A", k -&gt; new ArrayList&lt;&gt;()).add(1);</v>
+      </c>
+      <c r="C11" t="str" xml:space="preserve">
+        <v xml:space="preserve">当 value 是 List / Set / Map 时初始化：_x000d_
+map.computeIfAbsent(key, k -&gt; new ArrayList&lt;&gt;()).add(value);</v>
+      </c>
+      <c r="D11" t="str" xml:space="preserve">
+        <v xml:space="preserve">Map&lt;Character, List&lt;String&gt;&gt; map = new HashMap&lt;&gt;();_x000d_
+_x000d_
+String[] words = {"apple","ant","banana","boat"};_x000d_
+_x000d_
+for(String w : words){_x000d_
+    char c = w.charAt(0);_x000d_
+    map.computeIfAbsent(c, k -&gt; new ArrayList&lt;&gt;()).add(w);_x000d_
+}_x000d_
+_x000d_
+System.out.println(map);_x000d_
+------------------------------------_x000d_
+Map&lt;String, Integer&gt; count = new HashMap&lt;&gt;();_x000d_
+String[] words = {"apple", "banana", "apple", "orange", "banana"};_x000d_
+_x000d_
+for (String word : words) {_x000d_
+    count.computeIfAbsent(word, k -&gt; 0); // 如果没有 key，word就是关键词 ，值初始化为 0_x000d_
+    count.put(word, count.get(word) + 1); // 再 +1_x000d_
+}_x000d_
+_x000d_
+System.out.println(count);</v>
+      </c>
+    </row>
+    <row r="12" xml:space="preserve">
+      <c r="A12" t="str">
+        <v>map.putIfAbsent(key, value);</v>
+      </c>
+      <c r="B12" t="str">
+        <v>putIfAbsent只在不存在时放入，如果 key 已存在 → 不覆盖，初始化默认值</v>
+      </c>
+      <c r="C12" t="str" xml:space="preserve">
+        <v xml:space="preserve">需要你自己创建 value，_x000d_
+put() 会覆盖旧值。</v>
+      </c>
+      <c r="D12" t="str" xml:space="preserve">
+        <v xml:space="preserve">Map&lt;String, List&lt;Integer&gt;&gt; map = new HashMap&lt;&gt;();_x000d_
+map.putIfAbsent("A", new ArrayList&lt;&gt;());_x000d_
+map.get("A").add(1);_x000d_
+map.putIfAbsent("A", new ArrayList&lt;&gt;());_x000d_
+map.get("A").add(2);_x000d_
+System.out.println(map);//{A=[1, 2]}_x000d_
+------------------------------------------_x000d_
+Map&lt;String, Integer&gt; map = new HashMap&lt;&gt;();_x000d_
+map.put("A", 10);_x000d_
+map.putIfAbsent("A", 20);   // A 已存在，不会覆盖_x000d_
+map.putIfAbsent("B", 30);   // B 不存在，会添加_x000d_
+System.out.println(map);//{A=10, B=30} 因为A已经有了，所以即使加进去也没用</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>map.replace(key, oldVal, newVal)</v>
+      </c>
+      <c r="B13" t="str">
+        <v>替换指定 key 的值（如果值是 oldVal）</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>map.clear()</v>
+      </c>
+      <c r="B14" t="str">
+        <v>清空整个 Map</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>map.isEmpty()</v>
+      </c>
+      <c r="B15" t="str">
+        <v>判断是否为空</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>map.merge(key, value, BiFunction)</v>
+      </c>
+      <c r="B16" t="str">
+        <v>合并 value，例如累加频率</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>map.forEach((k,v) -&gt; {})</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Java 8 lambda 遍历</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>map.merge(key, 1, Integer::sum);</v>
+      </c>
+      <c r="B18" t="str">
+        <v>如果没有key，就1，有的话， 就累加sum</v>
+      </c>
+      <c r="C18" t="str">
+        <v>merge（最优雅计数法）计数 &amp; 累加，多用于字符统计，找重复元素</v>
+      </c>
+    </row>
+    <row r="19" xml:space="preserve">
+      <c r="A19" t="str">
+        <v>map.merge(key, 1, Integer::sum);</v>
+      </c>
+      <c r="B19" t="str">
+        <v>字符统计</v>
+      </c>
+      <c r="C19" t="str">
+        <v/>
+      </c>
+      <c r="D19" t="str" xml:space="preserve">
+        <v xml:space="preserve">Map&lt;Character, Integer&gt; count = new HashMap&lt;&gt;();_x000d_
+for (char c : "banana".toCharArray()) {_x000d_
+    count.merge(c, 1, Integer::sum);_x000d_
+}_x000d_
+System.out.println(count);//{b=1, a=3, n=2}_x000d_
+-------------------------------_x000d_
+if (map.merge(num, 1, Integer::sum) &gt; 1) {_x000d_
+    // duplicate_x000d_
+}</v>
+      </c>
+    </row>
+    <row r="20" xml:space="preserve">
+      <c r="A20" t="str">
+        <v>map.compute(key, (k, v) -&gt; v == null ? 1 : v + 1);</v>
+      </c>
+      <c r="B20" t="str">
+        <v>compute（万能函数），功能和 getOrDefault 类似，但更灵活。	统计频率</v>
+      </c>
+      <c r="C20" t="str" xml:space="preserve">
+        <v xml:space="preserve">如果 key 不存在 → value = 1_x000d_
+如果 key 已存在 → value + 1</v>
+      </c>
+      <c r="D20" t="str" xml:space="preserve">
+        <v xml:space="preserve">Map&lt;Character, Integer&gt; map = new HashMap&lt;&gt;();_x000d_
+_x000d_
+for(char c : "banana".toCharArray()){_x000d_
+    map.compute(c, (k, v) -&gt; v == null ? 1 : v + 1);_x000d_
+}_x000d_
+_x000d_
+System.out.println(map);//{b=1, a=3, n=2}</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D20"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D16"/>
+  <sheetData>
+    <row r="1" xml:space="preserve">
+      <c r="A1" t="str" xml:space="preserve">
+        <v xml:space="preserve">priorityqueue： 一个按优先级自动排序的队列_x000d_
+	•	不是 FIFO_x000d_
+	•	每次取出的都是 优先级最高的元素</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>方法</v>
+      </c>
+      <c r="B2" t="str">
+        <v>功能</v>
+      </c>
+      <c r="C2" t="str">
+        <v>备注</v>
+      </c>
+      <c r="D2" t="str">
+        <v>例子</v>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3" t="str">
+        <v>new PriorityQueue&lt;&gt;()</v>
+      </c>
+      <c r="B3" t="str">
+        <v>创建最小堆</v>
+      </c>
+      <c r="C3" t="str">
+        <v>默认 小顶堆</v>
+      </c>
+      <c r="D3" t="str" xml:space="preserve">
+        <v xml:space="preserve">PriorityQueue&lt;Integer&gt; pq = new PriorityQueue&lt;&gt;();_x000d_
+PriorityQueue&lt;Integer&gt; pq = new PriorityQueue&lt;&gt;((a,b) -&gt; count.get(a) - count.get(b));</v>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str">
+        <v>new PriorityQueue&lt;&gt;(Comparator.reverseOrder())</v>
+      </c>
+      <c r="B4" t="str">
+        <v>创建最大堆</v>
+      </c>
+      <c r="C4" t="str" xml:space="preserve">
+        <v xml:space="preserve">常用于 TopK｜_x000d_
+PriorityQueue&lt;Integer&gt; maxHeap =new PriorityQueue&lt;&gt;((a, b) -&gt; b - a);</v>
+      </c>
+      <c r="D4" t="str" xml:space="preserve">
+        <v xml:space="preserve">PriorityQueue&lt;Integer&gt; pq =_x000d_
+        new PriorityQueue&lt;&gt;(Comparator.reverseOrder());_x000d_
+_x000d_
+pq.offer(5);_x000d_
+pq.offer(2);_x000d_
+pq.offer(8);_x000d_
+852_x000d_
+System.out.println(pq.poll());//8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>offer(e)</v>
+      </c>
+      <c r="B5" t="str">
+        <v>添加元素</v>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v>pq.offer(5);</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>add(e)</v>
+      </c>
+      <c r="B6" t="str">
+        <v>添加元素与 offer 类似</v>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+      <c r="D6" t="str">
+        <v>pq.add(10);</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>peek()</v>
+      </c>
+      <c r="B7" t="str">
+        <v>查看堆顶</v>
+      </c>
+      <c r="C7" t="str">
+        <v>返回最小值，不删除</v>
+      </c>
+      <c r="D7" t="str">
+        <v>pq.peek();</v>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
+      <c r="A8" t="str">
+        <v>pq.poll();</v>
+      </c>
+      <c r="B8" t="str">
+        <v>取出堆顶,同时删除</v>
+      </c>
+      <c r="C8" t="str">
+        <v>删除并返回最小值</v>
+      </c>
+      <c r="D8" t="str" xml:space="preserve">
+        <v xml:space="preserve">PriorityQueue&lt;Integer&gt; pq = new PriorityQueue&lt;&gt;();_x000d_
+pq.offer(5);_x000d_
+pq.offer(2);_x000d_
+pq.offer(8);_x000d_
+System.out.println(pq.peek()); // 2_x000d_
+System.out.println(pq.poll()); // 2_x000d_
+System.out.println(pq.poll()); // 5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>remove()</v>
+      </c>
+      <c r="B9" t="str">
+        <v>删除堆顶,</v>
+      </c>
+      <c r="C9" t="str">
+        <v>空时会报错</v>
+      </c>
+      <c r="D9" t="str">
+        <v>pq.remove();</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>size()</v>
+      </c>
+      <c r="B10" t="str">
+        <v>当前元素数量</v>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+      <c r="D10" t="str">
+        <v>pq.size();</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>isEmpty()</v>
+      </c>
+      <c r="B11" t="str">
+        <v>是否为空</v>
+      </c>
+      <c r="C11" t="str">
+        <v/>
+      </c>
+      <c r="D11" t="str">
+        <v>pq.isEmpty();</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>clear()</v>
+      </c>
+      <c r="B12" t="str">
+        <v>清空队列</v>
+      </c>
+      <c r="C12" t="str">
+        <v/>
+      </c>
+      <c r="D12" t="str">
+        <v>pq.clear();</v>
+      </c>
+    </row>
+    <row r="13" xml:space="preserve">
+      <c r="A13" t="str">
+        <v>contains(x)</v>
+      </c>
+      <c r="B13" t="str" xml:space="preserve">
+        <v xml:space="preserve">是否存在元素_x000d_
+O(n)</v>
+      </c>
+      <c r="C13" t="str">
+        <v/>
+      </c>
+      <c r="D13" t="str">
+        <v>pq.contains(5);</v>
+      </c>
+    </row>
+    <row r="14" xml:space="preserve">
+      <c r="A14" t="str">
+        <v>如果要求第 K 小怎么办？</v>
+      </c>
+      <c r="B14" t="str">
+        <v/>
+      </c>
+      <c r="C14" t="str">
+        <v/>
+      </c>
+      <c r="D14" t="str" xml:space="preserve">
+        <v xml:space="preserve">PriorityQueue&lt;Integer&gt; pq =_x000d_
+        new PriorityQueue&lt;&gt;(Collections.reverseOrder());变成大顶堆"</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>PriorityQueue((a,b)-&gt;map.get(a)-map.get(b))</v>
+      </c>
+      <c r="B15" t="str">
+        <v>按 map value 排序，value小的在堆顶，升序</v>
+      </c>
+      <c r="C15" t="str">
+        <v/>
+      </c>
+      <c r="D15" t="str">
+        <v>PriorityQueue&lt;Integer&gt; pq =new PriorityQueue&lt;&gt;(Comparator.comparingInt(map::get));</v>
+      </c>
+    </row>
+    <row r="16" xml:space="preserve">
+      <c r="A16" t="str" xml:space="preserve">
+        <v xml:space="preserve">PriorityQueue&lt;Integer&gt; pq =_x000d_
+    new PriorityQueue&lt;&gt;((a,b) -&gt; map.get(b) - map.get(a));</v>
+      </c>
+      <c r="B16" t="str">
+        <v>按 map value 排序，value大的在堆顶，降序</v>
+      </c>
+      <c r="C16" t="str">
+        <v>PriorityQueue&lt;Integer&gt; pq = new PriorityQueue&lt;&gt;(Comparator.comparingInt(map::get));</v>
+      </c>
+      <c r="D16" t="str" xml:space="preserve">
+        <v xml:space="preserve">PriorityQueue&lt;Integer&gt; pq =_x000d_
+    new PriorityQueue&lt;&gt;(Comparator.comparingInt(map::get).reversed());</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D16"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D30"/>
+  <sheetData>
+    <row r="1" xml:space="preserve">
+      <c r="A1" t="str" xml:space="preserve">
+        <v xml:space="preserve">Stream：_x000d_
+Arrays.stream(nums);   // 数组_x000d_
+list.stream();         // 集合_x000d_
+Stream.of(1,2,3);      // 手动创建</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>方法</v>
+      </c>
+      <c r="B2" t="str">
+        <v>功能</v>
+      </c>
+      <c r="C2" t="str">
+        <v>备注</v>
+      </c>
+      <c r="D2" t="str">
+        <v>例子</v>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3" t="str">
+        <v>Stream.of()</v>
+      </c>
+      <c r="B3" t="str">
+        <v>手动创建</v>
+      </c>
+      <c r="C3" t="str">
+        <v>测试 / 临时数据</v>
+      </c>
+      <c r="D3" t="str" xml:space="preserve">
+        <v xml:space="preserve">Stream.of(1, 2, 3, 4)_x000d_
+.forEach(System.out::println);</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Arrays.stream(nums)</v>
+      </c>
+      <c r="B4" t="str">
+        <v>来源数组</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>list.stream()</v>
+      </c>
+      <c r="B5" t="str">
+        <v>来源集合</v>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6" t="str">
+        <v>reduce()</v>
+      </c>
+      <c r="B6" t="str">
+        <v>求和累加</v>
+      </c>
+      <c r="C6" t="str" xml:space="preserve">
+        <v xml:space="preserve">int sum = list.stream()_x000d_
+.reduce(0, (a,b) -&gt; a + b);</v>
+      </c>
+      <c r="D6" t="str" xml:space="preserve">
+        <v xml:space="preserve">int sum =_x000d_
+Stream.of(1,2,3,4)_x000d_
+.reduce(0, (a,b) -&gt; a + b);_x000d_
+System.out.println(sum); // 10</v>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
+      <c r="A7" t="str">
+        <v>.boxed().toList()</v>
+      </c>
+      <c r="B7" t="str">
+        <v>int[] → List</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Arrays.stream + boxed</v>
+      </c>
+      <c r="D7" t="str" xml:space="preserve">
+        <v xml:space="preserve">int[] nums = {1,2,3,4};_x000d_
+List&lt;Integer&gt; list =_x000d_
+Arrays.stream(nums)_x000d_
+.boxed().toList();_x000d_
+System.out.println(list); // [1,2,3,4]</v>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
+      <c r="A8" t="str">
+        <v>Arrays.asList()</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Integer[] → List</v>
+      </c>
+      <c r="C8" t="str">
+        <v>数组 → List       Arrays.asList</v>
+      </c>
+      <c r="D8" t="str" xml:space="preserve">
+        <v xml:space="preserve">Integer[] arr = {1,2,3};_x000d_
+List&lt;Integer&gt; list = Arrays.asList(arr);_x000d_
+System.out.println(list); // [1,2,3]</v>
+      </c>
+    </row>
+    <row r="9" xml:space="preserve">
+      <c r="A9" t="str">
+        <v>Arrays.asList</v>
+      </c>
+      <c r="B9" t="str">
+        <v>String → List</v>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str" xml:space="preserve">
+        <v xml:space="preserve">String s = "apple banana orange";_x000d_
+List&lt;String&gt; list =Arrays.asList(s.split(" "));_x000d_
+System.out.println(list); // [apple, banana, orange]</v>
+      </c>
+    </row>
+    <row r="10" xml:space="preserve">
+      <c r="A10" t="str" xml:space="preserve">
+        <v xml:space="preserve">Stream.of(1,2,3)_x000d_
+.toList();</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Stream → List</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Stream → List     toList()</v>
+      </c>
+      <c r="D10" t="str" xml:space="preserve">
+        <v xml:space="preserve">List&lt;Integer&gt; list =_x000d_
+Stream.of(1,2,3)_x000d_
+.toList();</v>
+      </c>
+    </row>
+    <row r="11" xml:space="preserve">
+      <c r="A11" t="str" xml:space="preserve">
+        <v xml:space="preserve">filter(n -&gt; n &gt; 2)_x000d_
+.boxed().toList();</v>
+      </c>
+      <c r="B11" t="str">
+        <v>filter 后转 List</v>
+      </c>
+      <c r="C11" t="str">
+        <v/>
+      </c>
+      <c r="D11" t="str" xml:space="preserve">
+        <v xml:space="preserve">List&lt;Integer&gt; list =_x000d_
+Arrays.stream(new int[]{1,2,3,4}) .filter(n -&gt; n &gt; 2)_x000d_
+.boxed().toList();System.out.println(list); // [3,4]</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>map转换</v>
+      </c>
+      <c r="B12" t="str">
+        <v>map（转换）</v>
+      </c>
+      <c r="C12" t="str">
+        <v>每个元素转换</v>
+      </c>
+      <c r="D12" t="str">
+        <v>list.stream().map(n -&gt; n * 2)</v>
+      </c>
+    </row>
+    <row r="13" xml:space="preserve">
+      <c r="A13" t="str">
+        <v>mapToInt</v>
+      </c>
+      <c r="B13" t="str">
+        <v>mapToInt（转基本类型）</v>
+      </c>
+      <c r="C13" t="str">
+        <v>转成 IntStream</v>
+      </c>
+      <c r="D13" t="str" xml:space="preserve">
+        <v xml:space="preserve">list.stream()_x000d_
+.mapToInt(Integer::intValue)</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>distinct</v>
+      </c>
+      <c r="B14" t="str">
+        <v>（去重）</v>
+      </c>
+      <c r="C14" t="str">
+        <v>保留顺序</v>
+      </c>
+      <c r="D14" t="str">
+        <v>list.stream().distinct()</v>
+      </c>
+    </row>
+    <row r="15" xml:space="preserve">
+      <c r="A15" t="str">
+        <v>sorted</v>
+      </c>
+      <c r="B15" t="str">
+        <v>（排序）</v>
+      </c>
+      <c r="C15" t="str">
+        <v/>
+      </c>
+      <c r="D15" t="str" xml:space="preserve">
+        <v xml:space="preserve">list.stream().sorted(); // 升序_x000d_
+list.stream().sorted((a,b) -&gt; b - a); // 降序</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>limit</v>
+      </c>
+      <c r="B16" t="str">
+        <v>（取前 K 个）</v>
+      </c>
+      <c r="C16" t="str">
+        <v/>
+      </c>
+      <c r="D16" t="str">
+        <v>list.stream().limit(3);</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>list.stream().skip(2);</v>
+      </c>
+      <c r="B17" t="str">
+        <v>skip（跳过前 n 个）</v>
+      </c>
+      <c r="C17" t="str">
+        <v/>
+      </c>
+      <c r="D17" t="str">
+        <v>list.stream().skip(2);</v>
+      </c>
+    </row>
+    <row r="18" xml:space="preserve">
+      <c r="A18" t="str">
+        <v>stream().collect</v>
+      </c>
+      <c r="B18" t="str">
+        <v/>
+      </c>
+      <c r="C18" t="str">
+        <v>java8</v>
+      </c>
+      <c r="D18" t="str" xml:space="preserve">
+        <v xml:space="preserve">list.stream()_x000d_
+.collect(Collectors.toList());</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>stream().count()</v>
+      </c>
+      <c r="B19" t="str">
+        <v>（计数）</v>
+      </c>
+      <c r="C19" t="str">
+        <v/>
+      </c>
+      <c r="D19" t="str">
+        <v>long count = list.stream().count();</v>
+      </c>
+    </row>
+    <row r="20" xml:space="preserve">
+      <c r="A20" t="str">
+        <v>findFirst</v>
+      </c>
+      <c r="B20" t="str">
+        <v/>
+      </c>
+      <c r="C20" t="str">
+        <v/>
+      </c>
+      <c r="D20" t="str" xml:space="preserve">
+        <v xml:space="preserve">list.stream().filter(n -&gt; n &gt; 2)_x000d_
+.findFirst().orElse(-1);</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Arrays.stream(nums).sum();</v>
+      </c>
+      <c r="B21" t="str">
+        <v>求合</v>
+      </c>
+      <c r="C21" t="str">
+        <v>IntStream 专属方法</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Arrays.stream(nums).max().getAsInt();</v>
+      </c>
+      <c r="B22" t="str">
+        <v>最大值</v>
+      </c>
+      <c r="C22" t="str">
+        <v>IntStream 专属方法</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Arrays.stream(nums).min().getAsInt();</v>
+      </c>
+      <c r="B23" t="str">
+        <v>最小值</v>
+      </c>
+      <c r="C23" t="str">
+        <v>IntStream 专属方法</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Arrays.stream(nums).average().getAsDouble();</v>
+      </c>
+      <c r="B24" t="str">
+        <v>求平均</v>
+      </c>
+      <c r="C24" t="str">
+        <v>IntStream 专属方法</v>
+      </c>
+    </row>
+    <row r="25" xml:space="preserve">
+      <c r="A25" t="str">
+        <v>Map + Stream</v>
+      </c>
+      <c r="B25" t="str">
+        <v>按 value 排序</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Map + Stream</v>
+      </c>
+      <c r="D25" t="str" xml:space="preserve">
+        <v xml:space="preserve">map.entrySet().stream()_x000d_
+.sorted((a,b) -&gt; b.getValue() - a.getValue()).toList();</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>map.keySet().stream().toList();</v>
+      </c>
+      <c r="B26" t="str">
+        <v>取 key</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>map.values().stream().toList();</v>
+      </c>
+      <c r="B27" t="str">
+        <v>取 value</v>
+      </c>
+    </row>
+    <row r="28" xml:space="preserve">
+      <c r="A28" t="str" xml:space="preserve">
+        <v xml:space="preserve">map.values()_x000d_
+.stream().sorted().toList();</v>
+      </c>
+      <c r="B28" t="str">
+        <v>map排序后转 List</v>
+      </c>
+      <c r="C28" t="str">
+        <v>默认升序</v>
+      </c>
+      <c r="D28" t="str" xml:space="preserve">
+        <v xml:space="preserve">List&lt;Integer&gt; sortedValues = map.values()_x000d_
+.stream().sorted().toList();_x000d_
+System.out.println(sortedValues);</v>
+      </c>
+    </row>
+    <row r="29" xml:space="preserve">
+      <c r="A29" t="str" xml:space="preserve">
+        <v xml:space="preserve">map.values()_x000d_
+.stream().map(String::valueOf).toList()</v>
+      </c>
+      <c r="B29" t="str">
+        <v>map → 其他类型（比如 String）</v>
+      </c>
+      <c r="C29" t="str">
+        <v/>
+      </c>
+      <c r="D29" t="str" xml:space="preserve">
+        <v xml:space="preserve">List&lt;String&gt; strValues = map.values()_x000d_
+.stream().map(String::valueOf).toList();_x000d_
+_x000d_
+System.out.println(strValues);//["3", "5", "2"]</v>
       </c>
     </row>
     <row r="30" xml:space="preserve">
       <c r="A30" t="str">
-        <v>Set&lt;String&gt; set = Arrays.stream(words).collect(Collectors.toSet());</v>
+        <v>.toList()</v>
       </c>
       <c r="B30" t="str">
-        <v>数组 → 流 → 去重 → Set</v>
+        <v>把 Stream 里的元素收集到一个新的 List 中</v>
       </c>
       <c r="C30" t="str">
-        <v/>
+        <v>toList() 是 Stream 的终止操作</v>
       </c>
       <c r="D30" t="str" xml:space="preserve">
-        <v xml:space="preserve">String[] words = {"apple", "banana", "apple", "orange"};
-Set&lt;String&gt; set = Arrays.stream(words).collect(Collectors.toSet());//["apple", "banana", "orange"]</v>
+        <v xml:space="preserve">List&lt;Integer&gt; list = List.of(1,2,3,4);_x000d_
+// 筛选大于 2 的元素_x000d_
+List&lt;Integer&gt; res = list.stream()_x000d_
+                        .filter(n -&gt; n &gt; 2)_x000d_
+                        .toList();_x000d_
+System.out.println(res); // [3,4]</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:D30"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D33"/>
   <sheetData>
     <row r="1" xml:space="preserve">
       <c r="A1" t="str" xml:space="preserve">
-        <v xml:space="preserve">priorityqueue： 一个按优先级自动排序的队列
-	•	不是 FIFO
-	•	每次取出的都是 优先级最高的元素</v>
+        <v xml:space="preserve">🔥 面试必记 5 个坑_x000d_
+_x000d_
+❗ Arrays.asList() → 不能 add/remove_x000d_
+❗ toArray() 默认是 Object[]_x000d_
+❗ int[] 不能直接 asList（会变一个元素）_x000d_
+❗ toList()（Java 16+）是 不可变_x000d_
+❗ List&lt;Integer&gt; ≠ int[]（需要 stream 转换）</v>
+      </c>
+      <c r="B1" t="str" xml:space="preserve">
+        <v xml:space="preserve">👉 集合转换核心就是三套工具：_x000d_
+Arrays.asList()_x000d_
+toArray()_x000d_
+stream()</v>
+      </c>
+      <c r="C1" t="str" xml:space="preserve">
+        <v xml:space="preserve">String[] → Set:new HashSet&lt;&gt;(Arrays.asList(arr))_x000d_
+int[] → Set:Arrays.stream(arr).boxed().collect(...)</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>方法</v>
+        <v>Java 数组 &amp; 集合互转速查表 方法</v>
       </c>
       <c r="B2" t="str">
         <v>功能</v>
@@ -878,652 +1827,317 @@
     </row>
     <row r="3" xml:space="preserve">
       <c r="A3" t="str">
-        <v>new PriorityQueue&lt;&gt;()</v>
+        <v xml:space="preserve"> List → 数组</v>
       </c>
       <c r="B3" t="str">
-        <v>创建最小堆</v>
+        <v>String List → String[]</v>
       </c>
       <c r="C3" t="str">
-        <v>默认 小顶堆</v>
+        <v>错误Object[] arr = list.toArray(); // 不能当 String[] 用</v>
       </c>
       <c r="D3" t="str" xml:space="preserve">
-        <v xml:space="preserve">PriorityQueue&lt;Integer&gt; pq = new PriorityQueue&lt;&gt;();
-PriorityQueue&lt;Integer&gt; pq = new PriorityQueue&lt;&gt;((a,b) -&gt; count.get(a) - count.get(b));</v>
+        <v xml:space="preserve">List&lt;String&gt; list = Arrays.asList("a", "b", "c");_x000d_
+String[] arr = list.toArray(new String[0]);</v>
       </c>
     </row>
     <row r="4" xml:space="preserve">
-      <c r="A4" t="str">
-        <v>new PriorityQueue&lt;&gt;(Comparator.reverseOrder())</v>
+      <c r="A4" t="str" xml:space="preserve">
+        <v xml:space="preserve"> 数组 → 不可修改 List_x000d_
+最常用：Arrays.asList()</v>
       </c>
       <c r="B4" t="str">
-        <v>创建最大堆</v>
+        <v>数组 → 不可修改List</v>
       </c>
       <c r="C4" t="str" xml:space="preserve">
-        <v xml:space="preserve">常用于 TopK｜
-PriorityQueue&lt;Integer&gt; maxHeap =new PriorityQueue&lt;&gt;((a, b) -&gt; b - a);</v>
+        <v xml:space="preserve">✅ 普通写法，⚠️ 不可增删（重点！_x000d_
+toList() 返回的也是 不可变 List</v>
       </c>
       <c r="D4" t="str" xml:space="preserve">
-        <v xml:space="preserve">PriorityQueue&lt;Integer&gt; pq =
-        new PriorityQueue&lt;&gt;(Comparator.reverseOrder());
-pq.offer(5);
-pq.offer(2);
-pq.offer(8);
-852
-System.out.println(pq.poll());//8</v>
+        <v xml:space="preserve">String[] arr = {"a", "b", "c"};_x000d_
+List&lt;String&gt; list = Arrays.asList(arr); 或者_x000d_
+String[] arr = {"a", "b", "c"};_x000d_
+List&lt;String&gt; list = Arrays.stream(arr).toList();</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>offer(e)</v>
+        <v xml:space="preserve"> 数组 -&gt; 可修改 List（推荐）</v>
       </c>
       <c r="B5" t="str">
-        <v>添加元素</v>
-      </c>
-      <c r="C5" t="str">
-        <v/>
+        <v xml:space="preserve">数组 -&gt; 可修改 List </v>
       </c>
       <c r="D5" t="str">
-        <v>pq.offer(5);</v>
-      </c>
-    </row>
-    <row r="6">
+        <v>List&lt;String&gt; list = new ArrayList&lt;&gt;(Arrays.asList(arr));</v>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
       <c r="A6" t="str">
-        <v>add(e)</v>
+        <v>基本类型数组int[] → 不可变List（重点坑🔥）</v>
       </c>
       <c r="B6" t="str">
-        <v>添加元素与 offer 类似</v>
-      </c>
-      <c r="C6" t="str">
-        <v/>
-      </c>
-      <c r="D6" t="str">
-        <v>pq.add(10);</v>
-      </c>
-    </row>
-    <row r="7">
+        <v>int[] → 不可变List</v>
+      </c>
+      <c r="C6" t="str" xml:space="preserve">
+        <v xml:space="preserve">错误：int[] arr = {1, 2, 3};_x000d_
+List&lt;int[]&gt; list = Arrays.asList(arr); // ❗只有一个元素</v>
+      </c>
+      <c r="D6" t="str" xml:space="preserve">
+        <v xml:space="preserve">int[] arr = {1, 2, 3};_x000d_
+List&lt;Integer&gt; list = Arrays.stream(arr)_x000d_
+    .boxed()_x000d_
+    .toList();</v>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
       <c r="A7" t="str">
-        <v>peek()</v>
+        <v>基本类型数组int[] →可变 List</v>
       </c>
       <c r="B7" t="str">
-        <v>查看堆顶</v>
-      </c>
-      <c r="C7" t="str">
-        <v>返回最小值，不删除</v>
-      </c>
-      <c r="D7" t="str">
-        <v>pq.peek();</v>
+        <v>int[] →可变 List</v>
+      </c>
+      <c r="D7" t="str" xml:space="preserve">
+        <v xml:space="preserve">int[] arr = {1, 2, 3};_x000d_
+List&lt;Integer&gt; list = new ArrayList&lt;&gt;(_x000d_
+    Arrays.stream(arr).boxed().toList()_x000d_
+);_x000d_
+_x000d_
+list.add(4); // ✅ 可以</v>
       </c>
     </row>
     <row r="8" xml:space="preserve">
       <c r="A8" t="str">
-        <v>pq.poll();</v>
+        <v>List → 基本类型数组</v>
       </c>
       <c r="B8" t="str">
-        <v>取出堆顶,同时删除</v>
-      </c>
-      <c r="C8" t="str">
-        <v>删除并返回最小值</v>
+        <v>List → int[]</v>
       </c>
       <c r="D8" t="str" xml:space="preserve">
-        <v xml:space="preserve">PriorityQueue&lt;Integer&gt; pq = new PriorityQueue&lt;&gt;();
-pq.offer(5);
-pq.offer(2);
-pq.offer(8);
-System.out.println(pq.peek()); // 2
-System.out.println(pq.poll()); // 2
-System.out.println(pq.poll()); // 5</v>
-      </c>
-    </row>
-    <row r="9">
+        <v xml:space="preserve">List&lt;Integer&gt; list = Arrays.asList(1, 2, 3);_x000d_
+int[] arr = list.stream()_x000d_
+    .mapToInt(Integer::intValue)_x000d_
+    .toArray();</v>
+      </c>
+    </row>
+    <row r="9" xml:space="preserve">
       <c r="A9" t="str">
-        <v>remove()</v>
+        <v>Set → List</v>
       </c>
       <c r="B9" t="str">
-        <v>删除堆顶,</v>
-      </c>
-      <c r="C9" t="str">
-        <v>空时会报错</v>
-      </c>
-      <c r="D9" t="str">
-        <v>pq.remove();</v>
-      </c>
-    </row>
-    <row r="10">
+        <v>Set → List</v>
+      </c>
+      <c r="D9" t="str" xml:space="preserve">
+        <v xml:space="preserve">Set&lt;String&gt; set = new HashSet&lt;&gt;(Arrays.asList("a", "b"));_x000d_
+List&lt;String&gt; list = new ArrayList&lt;&gt;(set);</v>
+      </c>
+    </row>
+    <row r="10" xml:space="preserve">
       <c r="A10" t="str">
-        <v>size()</v>
+        <v>List → Set（去重🔥）</v>
       </c>
       <c r="B10" t="str">
-        <v>当前元素数量</v>
-      </c>
-      <c r="C10" t="str">
-        <v/>
-      </c>
-      <c r="D10" t="str">
-        <v>pq.size();</v>
-      </c>
-    </row>
-    <row r="11">
+        <v>List → Set（去重🔥）</v>
+      </c>
+      <c r="D10" t="str" xml:space="preserve">
+        <v xml:space="preserve">List&lt;String&gt; list = Arrays.asList("a", "a", "b");_x000d_
+Set&lt;String&gt; set = new HashSet&lt;&gt;(list);</v>
+      </c>
+    </row>
+    <row r="11" xml:space="preserve">
       <c r="A11" t="str">
-        <v>isEmpty()</v>
+        <v>String数组 → Set</v>
       </c>
       <c r="B11" t="str">
-        <v>是否为空</v>
-      </c>
-      <c r="C11" t="str">
-        <v/>
-      </c>
-      <c r="D11" t="str">
-        <v>pq.isEmpty();</v>
+        <v>对象数组 → Set</v>
+      </c>
+      <c r="D11" t="str" xml:space="preserve">
+        <v xml:space="preserve">String[] arr = {"a", "b", "a"};_x000d_
+Set&lt;String&gt; set = new HashSet&lt;&gt;(Arrays.asList(arr));</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>clear()</v>
+        <v>Set → String数组</v>
       </c>
       <c r="B12" t="str">
-        <v>清空队列</v>
-      </c>
-      <c r="C12" t="str">
-        <v/>
+        <v>Set → 对象型数组</v>
       </c>
       <c r="D12" t="str">
-        <v>pq.clear();</v>
+        <v>String[] arr = set.toArray(new String[0]);</v>
       </c>
     </row>
     <row r="13" xml:space="preserve">
       <c r="A13" t="str">
-        <v>contains(x)</v>
-      </c>
-      <c r="B13" t="str" xml:space="preserve">
-        <v xml:space="preserve">是否存在元素
-O(n)</v>
-      </c>
-      <c r="C13" t="str">
-        <v/>
-      </c>
-      <c r="D13" t="str">
-        <v>pq.contains(5);</v>
-      </c>
-    </row>
-    <row r="14" xml:space="preserve">
-      <c r="A14" t="str">
-        <v>如果要求第 K 小怎么办？</v>
-      </c>
-      <c r="B14" t="str">
-        <v/>
-      </c>
-      <c r="C14" t="str">
-        <v/>
-      </c>
-      <c r="D14" t="str" xml:space="preserve">
-        <v xml:space="preserve">PriorityQueue&lt;Integer&gt; pq =
-        new PriorityQueue&lt;&gt;(Collections.reverseOrder());变成大顶堆"</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>PriorityQueue((a,b)-&gt;map.get(a)-map.get(b))</v>
-      </c>
-      <c r="B15" t="str">
-        <v>按 map value 排序，value小的在堆顶，升序</v>
-      </c>
-      <c r="C15" t="str">
-        <v/>
-      </c>
-      <c r="D15" t="str">
-        <v>PriorityQueue&lt;Integer&gt; pq =new PriorityQueue&lt;&gt;(Comparator.comparingInt(map::get));</v>
-      </c>
-    </row>
-    <row r="16" xml:space="preserve">
-      <c r="A16" t="str" xml:space="preserve">
-        <v xml:space="preserve">PriorityQueue&lt;Integer&gt; pq =
-    new PriorityQueue&lt;&gt;((a,b) -&gt; map.get(b) - map.get(a));</v>
-      </c>
-      <c r="B16" t="str">
-        <v>按 map value 排序，value大的在堆顶，降序</v>
-      </c>
-      <c r="C16" t="str">
-        <v>PriorityQueue&lt;Integer&gt; pq = new PriorityQueue&lt;&gt;(Comparator.comparingInt(map::get));</v>
-      </c>
-      <c r="D16" t="str" xml:space="preserve">
-        <v xml:space="preserve">PriorityQueue&lt;Integer&gt; pq =
-    new PriorityQueue&lt;&gt;(Comparator.comparingInt(map::get).reversed());</v>
+        <v>基本类型数组 -&gt; Set</v>
+      </c>
+      <c r="B13" t="str">
+        <v>int[]基本类型数组 -&gt; Set</v>
+      </c>
+      <c r="C13" t="str" xml:space="preserve">
+        <v xml:space="preserve">wrong: int[] arr = {1, 2, 3};_x000d_
+Set&lt;int[]&gt; set = new HashSet&lt;&gt;(Arrays.asList(arr)); _x000d_
+Set 只能存对象（Integer),不能存基本类型,.boxed() 👉 把 int 转成 Integer</v>
+      </c>
+      <c r="D13" t="str" xml:space="preserve">
+        <v xml:space="preserve">int[] arr = {1, 2, 3};_x000d_
+_x000d_
+Set&lt;Integer&gt; set = Arrays.stream(arr)_x000d_
+    .boxed()_x000d_
+    .collect(Collectors.toSet());</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D33"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:A34"/>
   <sheetData>
-    <row r="1" xml:space="preserve">
-      <c r="A1" t="str" xml:space="preserve">
-        <v xml:space="preserve">Stream：
-Arrays.stream(nums);   // 数组
-list.stream();         // 集合
-Stream.of(1,2,3);      // 手动创建</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>方法</v>
-      </c>
-      <c r="B2" t="str">
-        <v>功能</v>
-      </c>
-      <c r="C2" t="str">
-        <v>备注</v>
-      </c>
-      <c r="D2" t="str">
-        <v>例子</v>
-      </c>
-    </row>
-    <row r="3" xml:space="preserve">
+    <row r="1">
+      <c r="A1" t="str">
+        <v>import java.util.*;</v>
+      </c>
+    </row>
+    <row r="3">
       <c r="A3" t="str">
-        <v>Stream.of()</v>
-      </c>
-      <c r="B3" t="str">
-        <v>手动创建</v>
-      </c>
-      <c r="C3" t="str">
-        <v>测试 / 临时数据</v>
-      </c>
-      <c r="D3" t="str" xml:space="preserve">
-        <v xml:space="preserve">Stream.of(1, 2, 3, 4)
-.forEach(System.out::println);</v>
+        <v>class Solution {</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Arrays.stream(nums)</v>
-      </c>
-      <c r="B4" t="str">
-        <v>来源数组</v>
+        <v xml:space="preserve">    public int[] maxSlidingWindow(int[] nums, int k) {</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>list.stream()</v>
-      </c>
-      <c r="B5" t="str">
-        <v>来源集合</v>
-      </c>
-    </row>
-    <row r="6" xml:space="preserve">
+        <v xml:space="preserve">        int n = nums.length;</v>
+      </c>
+    </row>
+    <row r="6">
       <c r="A6" t="str">
-        <v>reduce()</v>
-      </c>
-      <c r="B6" t="str">
-        <v>求和累加</v>
-      </c>
-      <c r="C6" t="str" xml:space="preserve">
-        <v xml:space="preserve">int sum = list.stream()
-.reduce(0, (a,b) -&gt; a + b);</v>
-      </c>
-      <c r="D6" t="str" xml:space="preserve">
-        <v xml:space="preserve">int sum =
-Stream.of(1,2,3,4)
-.reduce(0, (a,b) -&gt; a + b);
-System.out.println(sum); // 10</v>
-      </c>
-    </row>
-    <row r="7" xml:space="preserve">
+        <v xml:space="preserve">        int[] res = new int[n - k + 1];</v>
+      </c>
+    </row>
+    <row r="7">
       <c r="A7" t="str">
-        <v>.boxed().toList()</v>
-      </c>
-      <c r="B7" t="str">
-        <v>int[] → List</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Arrays.stream + boxed</v>
-      </c>
-      <c r="D7" t="str" xml:space="preserve">
-        <v xml:space="preserve">int[] nums = {1,2,3,4};
-List&lt;Integer&gt; list =
-Arrays.stream(nums)
-.boxed().toList();
-System.out.println(list); // [1,2,3,4]</v>
-      </c>
-    </row>
-    <row r="8" xml:space="preserve">
-      <c r="A8" t="str">
-        <v>Arrays.asList()</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Integer[] → List</v>
-      </c>
-      <c r="C8" t="str">
-        <v>数组 → List       Arrays.asList</v>
-      </c>
-      <c r="D8" t="str" xml:space="preserve">
-        <v xml:space="preserve">Integer[] arr = {1,2,3};
-List&lt;Integer&gt; list = Arrays.asList(arr);
-System.out.println(list); // [1,2,3]</v>
-      </c>
-    </row>
-    <row r="9" xml:space="preserve">
+        <v xml:space="preserve">        int idx = 0;</v>
+      </c>
+    </row>
+    <row r="9">
       <c r="A9" t="str">
-        <v>Arrays.asList</v>
-      </c>
-      <c r="B9" t="str">
-        <v>String → List</v>
-      </c>
-      <c r="C9" t="str">
-        <v/>
-      </c>
-      <c r="D9" t="str" xml:space="preserve">
-        <v xml:space="preserve">String s = "apple banana orange";
-List&lt;String&gt; list =Arrays.asList(s.split(" "));
-System.out.println(list); // [apple, banana, orange]</v>
-      </c>
-    </row>
-    <row r="10" xml:space="preserve">
-      <c r="A10" t="str" xml:space="preserve">
-        <v xml:space="preserve">Stream.of(1,2,3)
-.toList();</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Stream → List</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Stream → List     toList()</v>
-      </c>
-      <c r="D10" t="str" xml:space="preserve">
-        <v xml:space="preserve">List&lt;Integer&gt; list =
-Stream.of(1,2,3)
-.toList();</v>
-      </c>
-    </row>
-    <row r="11" xml:space="preserve">
-      <c r="A11" t="str" xml:space="preserve">
-        <v xml:space="preserve">filter(n -&gt; n &gt; 2)
-.boxed().toList();</v>
-      </c>
-      <c r="B11" t="str">
-        <v>filter 后转 List</v>
-      </c>
-      <c r="C11" t="str">
-        <v/>
-      </c>
-      <c r="D11" t="str" xml:space="preserve">
-        <v xml:space="preserve">List&lt;Integer&gt; list =
-Arrays.stream(new int[]{1,2,3,4}) .filter(n -&gt; n &gt; 2)
-.boxed().toList();System.out.println(list); // [3,4]</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>map转换</v>
-      </c>
-      <c r="B12" t="str">
-        <v>map（转换）</v>
-      </c>
-      <c r="C12" t="str">
-        <v>每个元素转换</v>
-      </c>
-      <c r="D12" t="str">
-        <v>list.stream().map(n -&gt; n * 2)</v>
-      </c>
-    </row>
-    <row r="13" xml:space="preserve">
+        <v xml:space="preserve">        Deque&lt;Integer&gt; deque = new ArrayDeque&lt;&gt;();</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v xml:space="preserve">        for (int i = 0; i &lt; n; i++) {</v>
+      </c>
+    </row>
+    <row r="13">
       <c r="A13" t="str">
-        <v>mapToInt</v>
-      </c>
-      <c r="B13" t="str">
-        <v>mapToInt（转基本类型）</v>
-      </c>
-      <c r="C13" t="str">
-        <v>转成 IntStream</v>
-      </c>
-      <c r="D13" t="str" xml:space="preserve">
-        <v xml:space="preserve">list.stream()
-.mapToInt(Integer::intValue)</v>
+        <v xml:space="preserve">            // 1️⃣ 移除过期元素（窗口左边界外）</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>distinct</v>
-      </c>
-      <c r="B14" t="str">
-        <v>（去重）</v>
-      </c>
-      <c r="C14" t="str">
-        <v>保留顺序</v>
-      </c>
-      <c r="D14" t="str">
-        <v>list.stream().distinct()</v>
-      </c>
-    </row>
-    <row r="15" xml:space="preserve">
+        <v xml:space="preserve">            if (!deque.isEmpty() &amp;&amp; deque.peekFirst() == i - k) {</v>
+      </c>
+    </row>
+    <row r="15">
       <c r="A15" t="str">
-        <v>sorted</v>
-      </c>
-      <c r="B15" t="str">
-        <v>（排序）</v>
-      </c>
-      <c r="C15" t="str">
-        <v/>
-      </c>
-      <c r="D15" t="str" xml:space="preserve">
-        <v xml:space="preserve">list.stream().sorted(); // 升序
-list.stream().sorted((a,b) -&gt; b - a); // 降序</v>
+        <v xml:space="preserve">                deque.pollFirst();</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>limit</v>
-      </c>
-      <c r="B16" t="str">
-        <v>（取前 K 个）</v>
-      </c>
-      <c r="C16" t="str">
-        <v/>
-      </c>
-      <c r="D16" t="str">
-        <v>list.stream().limit(3);</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>list.stream().skip(2);</v>
-      </c>
-      <c r="B17" t="str">
-        <v>skip（跳过前 n 个）</v>
-      </c>
-      <c r="C17" t="str">
-        <v/>
-      </c>
-      <c r="D17" t="str">
-        <v>list.stream().skip(2);</v>
-      </c>
-    </row>
-    <row r="18" xml:space="preserve">
+        <v xml:space="preserve">            }</v>
+      </c>
+    </row>
+    <row r="18">
       <c r="A18" t="str">
-        <v>stream().collect</v>
-      </c>
-      <c r="B18" t="str">
-        <v/>
-      </c>
-      <c r="C18" t="str">
-        <v>java8</v>
-      </c>
-      <c r="D18" t="str" xml:space="preserve">
-        <v xml:space="preserve">list.stream()
-.collect(Collectors.toList());</v>
+        <v xml:space="preserve">            // 2️⃣ 维护单调递减（把小的都踢掉）</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>stream().count()</v>
-      </c>
-      <c r="B19" t="str">
-        <v>（计数）</v>
-      </c>
-      <c r="C19" t="str">
-        <v/>
-      </c>
-      <c r="D19" t="str">
-        <v>long count = list.stream().count();</v>
-      </c>
-    </row>
-    <row r="20" xml:space="preserve">
+        <v xml:space="preserve">            while (!deque.isEmpty() &amp;&amp; nums[i] &gt;= nums[deque.peekLast()]) {</v>
+      </c>
+    </row>
+    <row r="20">
       <c r="A20" t="str">
-        <v>findFirst</v>
-      </c>
-      <c r="B20" t="str">
-        <v/>
-      </c>
-      <c r="C20" t="str">
-        <v/>
-      </c>
-      <c r="D20" t="str" xml:space="preserve">
-        <v xml:space="preserve">list.stream().filter(n -&gt; n &gt; 2)
-.findFirst().orElse(-1);</v>
+        <v xml:space="preserve">                deque.pollLast();</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Arrays.stream(nums).sum();</v>
-      </c>
-      <c r="B21" t="str">
-        <v>求合</v>
-      </c>
-      <c r="C21" t="str">
-        <v>IntStream 专属方法</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>Arrays.stream(nums).max().getAsInt();</v>
-      </c>
-      <c r="B22" t="str">
-        <v>最大值</v>
-      </c>
-      <c r="C22" t="str">
-        <v>IntStream 专属方法</v>
+        <v xml:space="preserve">            }</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Arrays.stream(nums).min().getAsInt();</v>
-      </c>
-      <c r="B23" t="str">
-        <v>最小值</v>
-      </c>
-      <c r="C23" t="str">
-        <v>IntStream 专属方法</v>
+        <v xml:space="preserve">            // 3️⃣ 加入当前元素（索引）</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Arrays.stream(nums).average().getAsDouble();</v>
-      </c>
-      <c r="B24" t="str">
-        <v>求平均</v>
-      </c>
-      <c r="C24" t="str">
-        <v>IntStream 专属方法</v>
-      </c>
-    </row>
-    <row r="25" xml:space="preserve">
-      <c r="A25" t="str">
-        <v>Map + Stream</v>
-      </c>
-      <c r="B25" t="str">
-        <v>按 value 排序</v>
-      </c>
-      <c r="C25" t="str">
-        <v>Map + Stream</v>
-      </c>
-      <c r="D25" t="str" xml:space="preserve">
-        <v xml:space="preserve">map.entrySet().stream()
-.sorted((a,b) -&gt; b.getValue() - a.getValue()).toList();</v>
+        <v xml:space="preserve">            deque.offerLast(i);</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>map.keySet().stream().toList();</v>
-      </c>
-      <c r="B26" t="str">
-        <v>取 key</v>
+        <v xml:space="preserve">            // 4️⃣ 记录结果（窗口形成后）</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>map.values().stream().toList();</v>
-      </c>
-      <c r="B27" t="str">
-        <v>取 value</v>
-      </c>
-    </row>
-    <row r="28" xml:space="preserve">
-      <c r="A28" t="str" xml:space="preserve">
-        <v xml:space="preserve">map.values()
-.stream().sorted().toList();</v>
-      </c>
-      <c r="B28" t="str">
-        <v>map排序后转 List</v>
-      </c>
-      <c r="C28" t="str">
-        <v>默认升序</v>
-      </c>
-      <c r="D28" t="str" xml:space="preserve">
-        <v xml:space="preserve">List&lt;Integer&gt; sortedValues = map.values()
-.stream().sorted().toList();
-System.out.println(sortedValues);</v>
-      </c>
-    </row>
-    <row r="29" xml:space="preserve">
-      <c r="A29" t="str" xml:space="preserve">
-        <v xml:space="preserve">map.values()
-.stream().map(String::valueOf).toList()</v>
-      </c>
-      <c r="B29" t="str">
-        <v>map → 其他类型（比如 String）</v>
-      </c>
-      <c r="C29" t="str">
-        <v/>
-      </c>
-      <c r="D29" t="str" xml:space="preserve">
-        <v xml:space="preserve">List&lt;String&gt; strValues = map.values()
-.stream().map(String::valueOf).toList();
-System.out.println(strValues);//["3", "5", "2"]</v>
-      </c>
-    </row>
-    <row r="30" xml:space="preserve">
+        <v xml:space="preserve">            if (i &gt;= k - 1) {</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v xml:space="preserve">                res[idx++] = nums[deque.peekFirst()];</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v xml:space="preserve">            }</v>
+      </c>
+    </row>
+    <row r="30">
       <c r="A30" t="str">
-        <v>.toList()</v>
-      </c>
-      <c r="B30" t="str">
-        <v>把 Stream 里的元素收集到一个新的 List 中</v>
-      </c>
-      <c r="C30" t="str">
-        <v>toList() 是 Stream 的终止操作</v>
-      </c>
-      <c r="D30" t="str" xml:space="preserve">
-        <v xml:space="preserve">List&lt;Integer&gt; list = List.of(1,2,3,4);
-// 筛选大于 2 的元素
-List&lt;Integer&gt; res = list.stream()
-                        .filter(n -&gt; n &gt; 2)
-                        .toList();
-System.out.println(res); // [3,4]</v>
+        <v xml:space="preserve">        }</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v xml:space="preserve">        return res;</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v xml:space="preserve">    }</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>}</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D30"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A34"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D47"/>
+  <dimension ref="A1:D44"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1578,7 +2192,7 @@
         <v>List.of 不可修改</v>
       </c>
       <c r="D4" t="str" xml:space="preserve">
-        <v xml:space="preserve">List&lt;Integer&gt; list = List.of(1,2,3);
+        <v xml:space="preserve">List&lt;Integer&gt; list = List.of(1,2,3);_x000d_
 list.add(4); // ❌ 报错</v>
       </c>
     </row>
@@ -1590,16 +2204,16 @@
         <v/>
       </c>
       <c r="C5" t="str" xml:space="preserve">
-        <v xml:space="preserve">创建一个 List 的
-不可修改副本（immutable copy）,
+        <v xml:space="preserve">创建一个 List 的_x000d_
+不可修改副本（immutable copy）,_x000d_
 copy 是不可修改的</v>
       </c>
       <c r="D5" t="str" xml:space="preserve">
-        <v xml:space="preserve">List&lt;Integer&gt; list = new ArrayList&lt;&gt;();
-list.add(1);
-list.add(2);
-list.add(3);
-List&lt;Integer&gt; copy = List.copyOf(list);
+        <v xml:space="preserve">List&lt;Integer&gt; list = new ArrayList&lt;&gt;();_x000d_
+list.add(1);_x000d_
+list.add(2);_x000d_
+list.add(3);_x000d_
+List&lt;Integer&gt; copy = List.copyOf(list);_x000d_
 System.out.println(copy);</v>
       </c>
     </row>
@@ -1636,20 +2250,22 @@
         <v>addAll(Collection c)</v>
       </c>
       <c r="B8" t="str" xml:space="preserve">
-        <v xml:space="preserve">把另一个集合里
+        <v xml:space="preserve">把另一个集合里_x000d_
 的所有元素添加到当前集合中</v>
       </c>
       <c r="C8" t="str">
         <v/>
       </c>
       <c r="D8" t="str" xml:space="preserve">
-        <v xml:space="preserve">List&lt;Integer&gt; list1 = new ArrayList&lt;&gt;();
-list1.add(1);
-list1.add(2);
-List&lt;Integer&gt; list2 = new ArrayList&lt;&gt;();
-list2.add(3);
-list2.add(4);
-list1.addAll(list2);
+        <v xml:space="preserve">List&lt;Integer&gt; list1 = new ArrayList&lt;&gt;();_x000d_
+list1.add(1);_x000d_
+list1.add(2);_x000d_
+_x000d_
+List&lt;Integer&gt; list2 = new ArrayList&lt;&gt;();_x000d_
+list2.add(3);_x000d_
+list2.add(4);_x000d_
+_x000d_
+list1.addAll(list2);_x000d_
 System.out.println(list1);//[1, 2, 3, 4]</v>
       </c>
     </row>
@@ -1658,17 +2274,17 @@
         <v>addAll(int index, Collection c)</v>
       </c>
       <c r="B9" t="str" xml:space="preserve">
-        <v xml:space="preserve">把集合 c 的所有元素插入到
+        <v xml:space="preserve">把集合 c 的所有元素插入到_x000d_
  List 的指定位置 index</v>
       </c>
       <c r="C9" t="str" xml:space="preserve">
-        <v xml:space="preserve">返回值 true/false，
+        <v xml:space="preserve">返回值 true/false，_x000d_
 true → 成功插入</v>
       </c>
       <c r="D9" t="str" xml:space="preserve">
-        <v xml:space="preserve">List&lt;Integer&gt; list = new ArrayList&lt;&gt;(List.of(1,2,5,6));
-List&lt;Integer&gt; add = List.of(3,4);
-list.addAll(2, add);
+        <v xml:space="preserve">List&lt;Integer&gt; list = new ArrayList&lt;&gt;(List.of(1,2,5,6));_x000d_
+List&lt;Integer&gt; add = List.of(3,4);_x000d_
+list.addAll(2, add);_x000d_
 System.out.println(list);</v>
       </c>
     </row>
@@ -1963,7 +2579,7 @@
         <v/>
       </c>
       <c r="D30" t="str" xml:space="preserve">
-        <v xml:space="preserve">List&lt;Integer&gt; list = List.of(3, 5, 1, 7, 2);
+        <v xml:space="preserve">List&lt;Integer&gt; list = List.of(3, 5, 1, 7, 2);_x000d_
 int minVal = Collections.min(list);</v>
       </c>
     </row>
@@ -2020,12 +2636,12 @@
         <v>防止修改</v>
       </c>
       <c r="D34" t="str" xml:space="preserve">
-        <v xml:space="preserve">List&lt;Integer&gt; original = new ArrayList&lt;&gt;();
-original.add(1);
-original.add(2);
-original.add(3);
-List&lt;Integer&gt; copy = List.copyOf(original);
-System.out.println(copy);// 这个copy新的list是无法改变，
+        <v xml:space="preserve">List&lt;Integer&gt; original = new ArrayList&lt;&gt;();_x000d_
+original.add(1);_x000d_
+original.add(2);_x000d_
+original.add(3);_x000d_
+List&lt;Integer&gt; copy = List.copyOf(original);_x000d_
+System.out.println(copy);// 这个copy新的list是无法改变，_x000d_
 copy.add(4);  // 会抛出 UnsupportedOperationException</v>
       </c>
     </row>
@@ -2051,14 +2667,14 @@
         <v>滤波/条件筛选</v>
       </c>
       <c r="C36" t="str" xml:space="preserve">
-        <v xml:space="preserve">返回 可修改的 List（通常是 ArrayList）
-可以继续 add、remove 元素，
+        <v xml:space="preserve">返回 可修改的 List（通常是 ArrayList）_x000d_
+可以继续 add、remove 元素，_x000d_
 List&lt;String&gt; result = words.stream() .filter(s -&gt; s.length() &gt; 3).collect(Collectors.toList());</v>
       </c>
       <c r="D36" t="str" xml:space="preserve">
-        <v xml:space="preserve">List&lt;Integer&gt; list = List.of(1, 2, 3, 4, 5);
-List&lt;Integer&gt; result = list.stream()
-.filter(n -&gt; n &gt; 2) // 过滤大于 2 的元素
+        <v xml:space="preserve">List&lt;Integer&gt; list = List.of(1, 2, 3, 4, 5);_x000d_
+List&lt;Integer&gt; result = list.stream()_x000d_
+.filter(n -&gt; n &gt; 2) // 过滤大于 2 的元素_x000d_
 .toList();  // 返回不可变List，不能修改</v>
       </c>
     </row>
@@ -2067,15 +2683,15 @@
         <v>stream().distinct()</v>
       </c>
       <c r="B37" t="str" xml:space="preserve">
-        <v xml:space="preserve">返回一个去重后的新 Stream，
+        <v xml:space="preserve">返回一个去重后的新 Stream，_x000d_
 保留原顺序，不修改原集合</v>
       </c>
       <c r="C37" t="str" xml:space="preserve">
-        <v xml:space="preserve">Set 不保留顺序（HashSet）
+        <v xml:space="preserve">Set 不保留顺序（HashSet）_x000d_
 distinct() 保留顺序</v>
       </c>
       <c r="D37" t="str" xml:space="preserve">
-        <v xml:space="preserve">List&lt;Integer&gt; list = List.of(1, 2, 2, 3, 3, 3, 4);
+        <v xml:space="preserve">List&lt;Integer&gt; list = List.of(1, 2, 2, 3, 3, 3, 4);_x000d_
 List&lt;Integer&gt; unique = list.stream().distinct().toList();   // Java 16+ 或 .collect(Collectors.toList())</v>
       </c>
     </row>
@@ -2084,14 +2700,14 @@
         <v>stream().sorted()</v>
       </c>
       <c r="B38" t="str" xml:space="preserve">
-        <v xml:space="preserve">返回一个排序后的新 Stream，
+        <v xml:space="preserve">返回一个排序后的新 Stream，_x000d_
 默认升序，原集合不变</v>
       </c>
       <c r="C38" t="str">
         <v/>
       </c>
       <c r="D38" t="str" xml:space="preserve">
-        <v xml:space="preserve">List&lt;Integer&gt; sorted = list.stream().sorted()  // 自然升序
+        <v xml:space="preserve">List&lt;Integer&gt; sorted = list.stream().sorted()  // 自然升序_x000d_
  .toList();</v>
       </c>
     </row>
@@ -2106,9 +2722,11 @@
         <v>words.stream().sorted(Comparator.comparingInt(String::length)).toList();//可以用方法引用</v>
       </c>
       <c r="D39" t="str" xml:space="preserve">
-        <v xml:space="preserve">List&lt;String&gt; words = List.of("apple","banana","kiwi");
-List&lt;String&gt; sortedByLength = words.stream().sorted((a, b) -&gt; a.length() - b.length())  // 按长度升序
-.toList();
+        <v xml:space="preserve">List&lt;String&gt; words = List.of("apple","banana","kiwi");_x000d_
+_x000d_
+List&lt;String&gt; sortedByLength = words.stream().sorted((a, b) -&gt; a.length() - b.length())  // 按长度升序_x000d_
+.toList();_x000d_
+_x000d_
 System.out.println(sortedByLength);</v>
       </c>
     </row>
@@ -2120,7 +2738,7 @@
         <v>倒序。</v>
       </c>
       <c r="C40" t="str" xml:space="preserve">
-        <v xml:space="preserve">reverse = 翻面
+        <v xml:space="preserve">reverse = 翻面_x000d_
 sort(reverseOrder) = 排序（降序）</v>
       </c>
       <c r="D40" t="str">
@@ -2135,12 +2753,12 @@
         <v>List -&gt; String</v>
       </c>
       <c r="C41" t="str" xml:space="preserve">
-        <v xml:space="preserve">stream写法更灵活
-String res = list.stream()
+        <v xml:space="preserve">stream写法更灵活_x000d_
+String res = list.stream()_x000d_
       .collect(Collectors.joining(","));</v>
       </c>
       <c r="D41" t="str" xml:space="preserve">
-        <v xml:space="preserve">List&lt;String&gt; list = List.of("apple", "banana", "orange");
+        <v xml:space="preserve">List&lt;String&gt; list = List.of("apple", "banana", "orange");_x000d_
 String res = String.join(",", list);或者用</v>
       </c>
     </row>
@@ -2152,12 +2770,12 @@
         <v>list转String，直接 toString（简单但格式固定）</v>
       </c>
       <c r="C42" t="str" xml:space="preserve">
-        <v xml:space="preserve">特殊：无分隔符拼接
+        <v xml:space="preserve">特殊：无分隔符拼接_x000d_
 String res = String.join("", list); 输出结果：applebananaorange</v>
       </c>
       <c r="D42" t="str" xml:space="preserve">
-        <v xml:space="preserve">List&lt;Integer&gt; list = List.of(1,2,3);
-String res = list.toString();
+        <v xml:space="preserve">List&lt;Integer&gt; list = List.of(1,2,3);_x000d_
+String res = list.toString();_x000d_
 System.out.println(res); // [1, 2, 3]</v>
       </c>
     </row>
@@ -2169,8 +2787,8 @@
         <v/>
       </c>
       <c r="C43" t="str" xml:space="preserve">
-        <v xml:space="preserve">List&lt;String&gt; → String      String.join(",", list)
-List&lt;Integer&gt; → String     stream + map + joining
+        <v xml:space="preserve">List&lt;String&gt; → String      String.join(",", list)_x000d_
+List&lt;Integer&gt; → String     stream + map + joining_x000d_
 需要格式控制               Collectors.joining()</v>
       </c>
     </row>
@@ -2185,84 +2803,35 @@
         <v>需要先转 String，stream + map + joining</v>
       </c>
       <c r="D44" t="str" xml:space="preserve">
-        <v xml:space="preserve">List&lt;Integer&gt; list = List.of(1,2,3);
-String res = list.stream().map(String::valueOf)
-             .collect(Collectors.joining(","));
+        <v xml:space="preserve">List&lt;Integer&gt; list = List.of(1,2,3);_x000d_
+String res = list.stream().map(String::valueOf)_x000d_
+             .collect(Collectors.joining(","));_x000d_
 System.out.println(res); // 1,2,3</v>
       </c>
     </row>
-    <row r="45" xml:space="preserve">
-      <c r="A45" t="str">
-        <v>List&lt;String&gt; list = new ArrayList&lt;&gt;(Collections.nCopies(3, ""));</v>
-      </c>
-      <c r="B45" t="str">
-        <v>创建 List（已知长度）</v>
-      </c>
-      <c r="C45" t="str">
-        <v>要有元素 → 用 nCopies 或 add，new ArrayList&lt;&gt;(n) → 只是容量</v>
-      </c>
-      <c r="D45" t="str" xml:space="preserve">
-        <v xml:space="preserve">List&lt;Integer&gt; list = new ArrayList&lt;&gt;(Collections.nCopies(5, 0));
-list.set(2, 100);
-System.out.println(list); // [0, 0, 100, 0, 0]</v>
-      </c>
-    </row>
-    <row r="46" xml:space="preserve">
-      <c r="A46" t="str" xml:space="preserve">
-        <v xml:space="preserve">int[][] ans = new int[result.size()][];  // 1️⃣ 创建二维数组
-ans = result.toArray(ans);                // 2️⃣ List → 数组</v>
-      </c>
-      <c r="B46" t="str" xml:space="preserve">
-        <v xml:space="preserve">List 转成二维数组，List&lt;int[]&gt; → int[][]
-步骤：
-1. 创建 int[][]，第一维长度 = list.size()
-2. 每行 = list.get(i)</v>
-      </c>
-      <c r="C46" t="str">
-        <v>result 是一个 List&lt;int[]&gt;（List 中每个元素是一个数组）所以 ans.length = result.size()</v>
-      </c>
-      <c r="D46" t="str" xml:space="preserve">
-        <v xml:space="preserve">List&lt;int[]&gt; result = new ArrayList&lt;&gt;();
-result.add(new int[]{1,2});
-result.add(new int[]{3,4,5});
-result.add(new int[]{6});</v>
-      </c>
-    </row>
-    <row r="47" xml:space="preserve">
-      <c r="A47" t="str">
-        <v>list.toArray(new String[0])</v>
-      </c>
-      <c r="B47" t="str">
-        <v>List&lt;String&gt; → String[]</v>
-      </c>
-      <c r="C47" t="str">
-        <v/>
-      </c>
-      <c r="D47" t="str" xml:space="preserve">
-        <v xml:space="preserve">List&lt;Integer&gt; list = Arrays.asList(1, 2, 3);
-Integer[] arr = list.toArray(new Integer[0]);</v>
-      </c>
-    </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D47"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D44"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D12"/>
   <sheetData>
     <row r="1" xml:space="preserve">
       <c r="A1" t="str" xml:space="preserve">
-        <v xml:space="preserve">Stack&lt;Integer&gt; stack = new Stack&lt;&gt;(); 
-Deque 当 Stack 用：
-Deque&lt;Integer&gt; stack = new ArrayDeque&lt;&gt;();
-后进先出，peek = 看顶，
-pop = 拿顶，search = 从顶往下找
-Stack 是 legacy 类（历史遗留）
-2.方法是 synchronized → 性能差
+        <v xml:space="preserve">Stack&lt;Integer&gt; stack = new Stack&lt;&gt;(); _x000d_
+Deque 当 Stack 用：_x000d_
+Deque&lt;Integer&gt; stack = new ArrayDeque&lt;&gt;();_x000d_
+后进先出，peek = 看顶，_x000d_
+pop = 拿顶，search = 从顶往下找</v>
+      </c>
+      <c r="B1" t="str" xml:space="preserve">
+        <v xml:space="preserve">Stack 是 legacy 类（历史遗留）_x000d_
+2.方法是 synchronized → 性能差_x000d_
 3.官方推荐用 Deque双端队列 替代</v>
       </c>
     </row>
@@ -2291,7 +2860,7 @@
         <v>底 → [1, 2] ← 栈顶</v>
       </c>
       <c r="D3" t="str" xml:space="preserve">
-        <v xml:space="preserve">stack.push(1);stack.push(2);
+        <v xml:space="preserve">stack.push(1);stack.push(2);_x000d_
 //[1, 2]</v>
       </c>
     </row>
@@ -2300,17 +2869,17 @@
         <v>pop()</v>
       </c>
       <c r="B4" t="str" xml:space="preserve">
-        <v xml:space="preserve">出栈,stack.pop(); 
+        <v xml:space="preserve">出栈,stack.pop(); _x000d_
 // pop 空栈,可能报错</v>
       </c>
       <c r="C4" t="str" xml:space="preserve">
-        <v xml:space="preserve">删除并返回栈顶元素
-原: [1,2], pop → 2
+        <v xml:space="preserve">删除并返回栈顶元素_x000d_
+原: [1,2], pop → 2_x000d_
 剩: [1]</v>
       </c>
       <c r="D4" t="str" xml:space="preserve">
-        <v xml:space="preserve">if(!stack.isEmpty()){
-    stack.pop();
+        <v xml:space="preserve">if(!stack.isEmpty()){_x000d_
+    stack.pop();_x000d_
 }</v>
       </c>
     </row>
@@ -2335,9 +2904,6 @@
       <c r="B6" t="str">
         <v>是否为空</v>
       </c>
-      <c r="C6" t="str">
-        <v/>
-      </c>
       <c r="D6" t="str">
         <v>stack.isEmpty();</v>
       </c>
@@ -2358,15 +2924,15 @@
         <v>返回从栈顶开始的位置（1-based）</v>
       </c>
       <c r="C8" t="str" xml:space="preserve">
-        <v xml:space="preserve">底 → [1, 2, 3] ← 栈顶，
+        <v xml:space="preserve">底 → [1, 2, 3] ← 栈顶，_x000d_
 找不到返回-1</v>
       </c>
       <c r="D8" t="str" xml:space="preserve">
-        <v xml:space="preserve">Stack&lt;Integer&gt; stack = new Stack&lt;&gt;();
-stack.push(1);
-stack.push(2);
-stack.push(3);
-int pos = stack.search(2);
+        <v xml:space="preserve">Stack&lt;Integer&gt; stack = new Stack&lt;&gt;();_x000d_
+stack.push(1);_x000d_
+stack.push(2);_x000d_
+stack.push(3);_x000d_
+int pos = stack.search(2);_x000d_
 System.out.println(pos);</v>
       </c>
     </row>
@@ -2374,19 +2940,13 @@
       <c r="A9" t="str">
         <v>逆序（用栈）</v>
       </c>
-      <c r="B9" t="str">
-        <v/>
-      </c>
-      <c r="C9" t="str">
-        <v/>
-      </c>
       <c r="D9" t="str" xml:space="preserve">
-        <v xml:space="preserve">Stack&lt;Integer&gt; stack = new Stack&lt;&gt;();
-for(int n : nums){
-    stack.push(n);
-}
-while(!stack.isEmpty()){
-System.out.println(stack.pop());
+        <v xml:space="preserve">Stack&lt;Integer&gt; stack = new Stack&lt;&gt;();_x000d_
+for(int n : nums){_x000d_
+    stack.push(n);_x000d_
+}_x000d_
+while(!stack.isEmpty()){_x000d_
+System.out.println(stack.pop());_x000d_
 }//输出2，因为从栈顶往下找，base从1</v>
       </c>
     </row>
@@ -2402,9 +2962,6 @@
       </c>
     </row>
     <row r="11" xml:space="preserve">
-      <c r="A11" t="str">
-        <v/>
-      </c>
       <c r="B11" t="str">
         <v>当队列用先进先出（FIFO）</v>
       </c>
@@ -2412,85 +2969,35 @@
         <v>不能存 null， 没有 search()</v>
       </c>
       <c r="D11" t="str" xml:space="preserve">
-        <v xml:space="preserve">dq.offer(1);
-dq.offer(2);
-dq.poll(); // 1
+        <v xml:space="preserve">dq.offer(1);_x000d_
+dq.offer(2);_x000d_
+dq.poll(); // 1_x000d_
 dq.peek(); // 2</v>
       </c>
     </row>
     <row r="12" xml:space="preserve">
       <c r="A12" t="str" xml:space="preserve">
-        <v xml:space="preserve">dq.offerFirst(1);  // 头插
-dq.offerLast(2);   // 尾插
-addLast(x) // 尾部插入
-removeLast() // 删除尾部
-pollLast() // 删除尾部
-peekLast() // 查看尾部
-dq.pollFirst();    // 头出
-dq.pollLast();     // 尾出
-peekFirst().  //查看头部
-queue.peek() → 头
-queue.poll() → 头（并删除）
-queue.remove() = 删除“队头”（最前面的元素）</v>
-      </c>
-      <c r="B12" t="str" xml:space="preserve">
-        <v xml:space="preserve">双端操作（Deque 精髓） 
-pollFirst() :删除头部（空返回 null）</v>
-      </c>
-    </row>
-    <row r="13" xml:space="preserve">
-      <c r="A13" t="str" xml:space="preserve">
-        <v xml:space="preserve">deque.offerLast(1);
-deque.offerLast(2);
-deque.pollFirst(); // 1</v>
-      </c>
-      <c r="B13" t="str">
-        <v>作为队列（FIFO）👉 先进先出</v>
-      </c>
-    </row>
-    <row r="14" xml:space="preserve">
-      <c r="A14" t="str" xml:space="preserve">
-        <v xml:space="preserve">deque.push(1);   // = addFirst
-deque.push(2);
-deque.pop();     // 2</v>
-      </c>
-      <c r="B14" t="str">
-        <v>作为栈（LIFO） 后进先出</v>
-      </c>
-      <c r="C14" t="str" xml:space="preserve">
-        <v xml:space="preserve">用于滑动窗口最大值 / 最小值。	把小的都踢掉（没用了）
-	•	保证队列是“单调的”</v>
-      </c>
-      <c r="D14" t="str" xml:space="preserve">
-        <v xml:space="preserve">while (!deque.isEmpty() &amp;&amp; nums[deque.peekLast()] &lt; nums[i]) {
-    deque.pollLast(); // 保持单调递减
-}
-deque.offerLast(i);</v>
-      </c>
-    </row>
-    <row r="15" xml:space="preserve">
-      <c r="A15" t="str" xml:space="preserve">
-        <v xml:space="preserve">窗口左边界 = i - k + 1
-窗口范围 = [i - k + 1, i]</v>
-      </c>
-      <c r="B15" t="str">
-        <v>k是窗口大小比如3个元素长度</v>
-      </c>
-      <c r="C15" t="str" xml:space="preserve">
-        <v xml:space="preserve">从尾部删，维护单调性（淘汰“没用的数”）
-从头部删，移除“过期的数”</v>
+        <v xml:space="preserve">dq.offerFirst(1);  // 头插_x000d_
+dq.offerLast(2);   // 尾插_x000d_
+_x000d_
+dq.pollFirst();    // 头出_x000d_
+dq.pollLast();     // 尾出</v>
+      </c>
+      <c r="B12" t="str">
+        <v>双端操作（Deque 精髓）</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D12"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D47"/>
+  <dimension ref="A1:D42"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2511,17 +3018,17 @@
         <v>str.contains(substring)</v>
       </c>
       <c r="B2" t="str" xml:space="preserve">
-        <v xml:space="preserve">判断字符串是否包含某个子字符串
+        <v xml:space="preserve">判断字符串是否包含某个子字符串_x000d_
 返回 boolean</v>
       </c>
       <c r="C2" t="str">
         <v/>
       </c>
       <c r="D2" t="str" xml:space="preserve">
-        <v xml:space="preserve">String str = "hello world";
-System.out.println(str.contains("java"));//输出false
-if (s.contains("abc")) { }
-if (s.contains(" ")) { }    // 是否有空格
+        <v xml:space="preserve">String str = "hello world";_x000d_
+System.out.println(str.contains("java"));//输出false_x000d_
+if (s.contains("abc")) { }_x000d_
+if (s.contains(" ")) { }    // 是否有空格_x000d_
 if (s.contains(".")) { }    // 是否有点</v>
       </c>
     </row>
@@ -2592,9 +3099,9 @@
         <v>常用回文判断，字符统计</v>
       </c>
       <c r="D7" t="str" xml:space="preserve">
-        <v xml:space="preserve">方法1：charAt
-for(int i=0;i&lt;s.length();i++){
-    char c = s.charAt(i);
+        <v xml:space="preserve">方法1：charAt_x000d_
+for(int i=0;i&lt;s.length();i++){_x000d_
+    char c = s.charAt(i);_x000d_
 }</v>
       </c>
     </row>
@@ -2609,8 +3116,8 @@
         <v/>
       </c>
       <c r="D8" t="str" xml:space="preserve">
-        <v xml:space="preserve">方法2：toCharArray（更快）
-String s = "hello";
+        <v xml:space="preserve">方法2：toCharArray（更快）_x000d_
+String s = "hello";_x000d_
 char[] arr = s.toCharArray();//['h','e','l','l','o']</v>
       </c>
     </row>
@@ -2674,19 +3181,16 @@
       <c r="A13" t="str">
         <v>substring(begin)</v>
       </c>
-      <c r="B13" t="str" xml:space="preserve">
-        <v xml:space="preserve">截取从 begin 到末尾，substring(beginIndex) 安全规则：
-✔ 0 &lt;= beginIndex &lt;= length()
-✔ beginIndex == length() → 返回 ""
-✔ beginIndex &gt; length() → 越界异常</v>
+      <c r="B13" t="str">
+        <v>截取从 begin 到末尾</v>
       </c>
       <c r="C13" t="str" xml:space="preserve">
-        <v xml:space="preserve">从索引 6 开始，截取到字符串结尾，
+        <v xml:space="preserve">从索引 6 开始，截取到字符串结尾，_x000d_
 返回的是 新的字符串。</v>
       </c>
       <c r="D13" t="str" xml:space="preserve">
-        <v xml:space="preserve">String s = "hello world";
-String sub = s.substring(6);
+        <v xml:space="preserve">String s = "hello world";_x000d_
+String sub = s.substring(6);_x000d_
 System.out.println(sub);//world</v>
       </c>
     </row>
@@ -2708,31 +3212,30 @@
       <c r="A15" t="str">
         <v>split(regex)</v>
       </c>
-      <c r="B15" t="str" xml:space="preserve">
-        <v xml:space="preserve">分割字符串，字符串 → 数组
-split 使用的是正则表达式，像 "." 这样的字符需要用 Pattern.quote 转义，否则会匹配所有字符导致结果错误</v>
+      <c r="B15" t="str">
+        <v>分割字符串，字符串 → 数组</v>
       </c>
       <c r="C15" t="str" xml:space="preserve">
-        <v xml:space="preserve">按空格 " " 把字符串拆分成
-多个字符串，返回 String[] 数组。用正则更好：String s = "I  love   Java";
+        <v xml:space="preserve">按空格 " " 把字符串拆分成_x000d_
+多个字符串，返回 String[] 数组。用正则更好：String s = "I  love   Java";_x000d_
 String[] arr = s.split("\\s+");</v>
       </c>
       <c r="D15" t="str" xml:space="preserve">
-        <v xml:space="preserve">String s = "I love Java";
-String[] arr = s.split(" ");
+        <v xml:space="preserve">String s = "I love Java";_x000d_
+String[] arr = s.split(" ");_x000d_
 System.out.println(Arrays.toString(arr));//[I, love, Java]</v>
       </c>
     </row>
     <row r="16" xml:space="preserve">
       <c r="A16" t="str">
-        <v>String.join(delimiter, list) 分隔符，要拼接的字符串集合or array</v>
+        <v>String.join(delimiter, list) 分隔符，要拼接的字符串集合</v>
       </c>
       <c r="B16" t="str" xml:space="preserve">
-        <v xml:space="preserve">数组/List 拼接成 字符串
+        <v xml:space="preserve">数组/List 拼接成 字符串_x000d_
 返回string</v>
       </c>
       <c r="C16" t="str">
-        <v>String.join(分隔符, 集合/数组)</v>
+        <v/>
       </c>
       <c r="D16" t="str">
         <v>List&lt;String&gt; list = Arrays.asList("2026", "03", "15");String result = String.join("-", list);System.out.println(result);//2026-03-15</v>
@@ -2743,7 +3246,7 @@
         <v>replace()</v>
       </c>
       <c r="B17" t="str">
-        <v>替换字符，String.replace() 会返回一个新的 String</v>
+        <v>替换字符</v>
       </c>
       <c r="C17" t="str">
         <v>把l 换成x</v>
@@ -2763,9 +3266,9 @@
         <v/>
       </c>
       <c r="D18" t="str" xml:space="preserve">
-        <v xml:space="preserve">s.replaceAll("[aeiou]", "*"); 把所有元音替换成*.
-s.replaceAll("\\s","")
-s.replaceAll("\\d", "");删除所有数字，
+        <v xml:space="preserve">s.replaceAll("[aeiou]", "*"); 把所有元音替换成*._x000d_
+s.replaceAll("\\s","")_x000d_
+s.replaceAll("\\d", "");删除所有数字，_x000d_
 s.replaceAll("[^a-zA-Z]", "");只保留字母</v>
       </c>
     </row>
@@ -2780,7 +3283,7 @@
         <v>s.trim()</v>
       </c>
     </row>
-    <row r="20" xml:space="preserve">
+    <row r="20">
       <c r="A20" t="str">
         <v>toLowerCase()</v>
       </c>
@@ -2788,11 +3291,10 @@
         <v>转小写</v>
       </c>
       <c r="C20" t="str">
-        <v>返回一个新的字符串</v>
-      </c>
-      <c r="D20" t="str" xml:space="preserve">
-        <v xml:space="preserve">String str = "Hello World!";
-String lower = str.toLowerCase()</v>
+        <v/>
+      </c>
+      <c r="D20" t="str">
+        <v>"HELLO".toLowerCase()</v>
       </c>
     </row>
     <row r="21">
@@ -2839,7 +3341,7 @@
         <v>String转数字,String → int</v>
       </c>
       <c r="C24" t="str" xml:space="preserve">
-        <v xml:space="preserve">parseInt 返回基本类型，
+        <v xml:space="preserve">parseInt 返回基本类型，_x000d_
 valueOf 返回对象。</v>
       </c>
       <c r="D24" t="str">
@@ -2857,7 +3359,8 @@
         <v>返回的是 对象 Integer。</v>
       </c>
       <c r="D25" t="str" xml:space="preserve">
-        <v xml:space="preserve">String s = "123";
+        <v xml:space="preserve">String s = "123";_x000d_
+_x000d_
 Integer n = Integer.valueOf(s);</v>
       </c>
     </row>
@@ -2869,13 +3372,13 @@
         <v>将任意类型转换为字符串。</v>
       </c>
       <c r="C26" t="str" xml:space="preserve">
-        <v xml:space="preserve">123 → "123"
-true → "true"
+        <v xml:space="preserve">123 → "123"_x000d_
+true → "true"_x000d_
 'A' → "A"</v>
       </c>
       <c r="D26" t="str" xml:space="preserve">
-        <v xml:space="preserve">int n=123;
-String s = String.valueOf(n);
+        <v xml:space="preserve">int n=123;_x000d_
+String s = String.valueOf(n);_x000d_
 System.out.println(s);// "123"</v>
       </c>
     </row>
@@ -2893,14 +3396,12 @@
         <v>String b = Integer.toString(123);</v>
       </c>
     </row>
-    <row r="28" xml:space="preserve">
-      <c r="A28" t="str" xml:space="preserve">
-        <v xml:space="preserve">stringbuilder.append("hi")
-sb.append(word, 0, word.length() - 1).append(" ");</v>
-      </c>
-      <c r="B28" t="str" xml:space="preserve">
-        <v xml:space="preserve">拼接字符
-或者</v>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>stringbuilder.append("hi")</v>
+      </c>
+      <c r="B28" t="str">
+        <v>拼接字符</v>
       </c>
     </row>
     <row r="29">
@@ -2922,8 +3423,8 @@
         <v>String是不可变的。</v>
       </c>
       <c r="D30" t="str" xml:space="preserve">
-        <v xml:space="preserve">StringBuilder sb = new StringBuilder("abcdef");
-sb.delete(1, 3);
+        <v xml:space="preserve">StringBuilder sb = new StringBuilder("abcdef");_x000d_
+sb.delete(1, 3);_x000d_
 System.out.println(sb)//adef</v>
       </c>
     </row>
@@ -2935,12 +3436,12 @@
         <v>删除单个字符</v>
       </c>
       <c r="C31" t="str" xml:space="preserve">
-        <v xml:space="preserve">删除最后一个字符：
+        <v xml:space="preserve">删除最后一个字符：_x000d_
 sb.deleteCharAt(sb.length() - 1);</v>
       </c>
       <c r="D31" t="str" xml:space="preserve">
-        <v xml:space="preserve">StringBuilder sb = new StringBuilder("hello");
-sb.deleteCharAt(1);
+        <v xml:space="preserve">StringBuilder sb = new StringBuilder("hello");_x000d_
+sb.deleteCharAt(1);_x000d_
 System.out.println(sb); //hllo</v>
       </c>
     </row>
@@ -2955,7 +3456,7 @@
         <v>它直接修改原对象，不会创建新对象。</v>
       </c>
       <c r="D32" t="str" xml:space="preserve">
-        <v xml:space="preserve">String reversed = new StringBuilder("world").reverse().toString();
+        <v xml:space="preserve">String reversed = new StringBuilder("world").reverse().toString();_x000d_
 System.out.println(reversed);//dlrow</v>
       </c>
     </row>
@@ -2977,7 +3478,7 @@
     </row>
     <row r="35" xml:space="preserve">
       <c r="A35" t="str" xml:space="preserve">
-        <v xml:space="preserve">StringBuilder sb = new StringBuilder("Hello");
+        <v xml:space="preserve">StringBuilder sb = new StringBuilder("Hello");_x000d_
 String s = sb.toString();</v>
       </c>
       <c r="B35" t="str">
@@ -3082,407 +3583,332 @@
         <v>有（synchronized）</v>
       </c>
     </row>
-    <row r="43" xml:space="preserve">
-      <c r="A43" t="str">
-        <v>stringbuilder.setCharAt(index，character)</v>
-      </c>
-      <c r="B43" t="str">
-        <v>修改某一位字符（只能用于 StringBuilder）</v>
-      </c>
-      <c r="C43" t="str">
-        <v>返回 void，不能赋值。setCharAt 是 Java 里 StringBuilder / StringBuffer 的方法</v>
-      </c>
-      <c r="D43" t="str" xml:space="preserve">
-        <v xml:space="preserve">StringBuilder sb = new StringBuilder("hello");
-sb.setCharAt(1, 'a');
-System.out.println(sb);//hallo</v>
-      </c>
-    </row>
-    <row r="44" xml:space="preserve">
-      <c r="A44" t="str">
-        <v>a.compareTo(b)/compareToIgnoreCase（忽略大小写）</v>
-      </c>
-      <c r="B44" t="str" xml:space="preserve">
-        <v xml:space="preserve">··返回 负数 → 当前字符串小于 anotherString
-··返回 0 → 两个字符串相等
-··返回 正数 → 当前字符串大于 anotherString</v>
-      </c>
-      <c r="C44" t="str">
-        <v/>
-      </c>
-      <c r="D44" t="str" xml:space="preserve">
-        <v xml:space="preserve">String x = "abc";
-String y = "abd";
-System.out.println(x.compareTo(y)); // -1 → 因为 'c' &lt; 'd'</v>
-      </c>
-    </row>
-    <row r="45" xml:space="preserve">
-      <c r="A45" t="str">
-        <v>sb.append(word, 0, word.length() - 1);</v>
-      </c>
-      <c r="B45" t="str" xml:space="preserve">
-        <v xml:space="preserve">等价于：
-sb.append(word.substring(0, word.length() - 1));</v>
-      </c>
-      <c r="C45" t="str">
-        <v>append(字符串, 起始下标, 结束下标)</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="str">
-        <v>String arr[] = words.get(i).split("[" + separator + "]");</v>
-      </c>
-      <c r="B46" t="str">
-        <v>[.]  → 表示匹配字符 . 本身</v>
-      </c>
-      <c r="C46" t="str">
-        <v>[.] = 只匹配 "."</v>
-      </c>
-      <c r="D46" t="str">
-        <v>"one.two".split("[.]")</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="str">
-        <v>String sp = Pattern.quote(String.valueOf(separator));</v>
-      </c>
-      <c r="B47" t="str">
-        <v>把char变成string，并匹配。不然"."会误以为正则表达</v>
-      </c>
-    </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D47"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D42"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D23"/>
-  <sheetData>
-    <row r="1" xml:space="preserve">
-      <c r="A1" t="str" xml:space="preserve">
-        <v xml:space="preserve">char 本质是一个整数（Unicode 编码）
-运算时会自动提升为 int（类型提升）
-小于 int 的类型（byte / short / char）参与运算 → 自动转成 int
-char 比较按 Unicode：'a' &gt; 'A'  // true
-char a = 'A'; // 65
-char b = 'B'; // 66
-int result = a + b;</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>方法</v>
-      </c>
-      <c r="B2" t="str">
-        <v>功能</v>
-      </c>
-      <c r="C2" t="str">
-        <v>备注</v>
-      </c>
-      <c r="D2" t="str">
-        <v>例子</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>int n = c - '0'</v>
-      </c>
-      <c r="B3" t="str">
-        <v>char变成int</v>
-      </c>
-      <c r="C3" t="str">
-        <v/>
-      </c>
-      <c r="D3" t="str">
-        <v>char c = '7';int n = c - '0';   // 7</v>
-      </c>
-    </row>
-    <row r="4" xml:space="preserve">
-      <c r="A4" t="str" xml:space="preserve">
-        <v xml:space="preserve">char c = (char) (n + '0');
-ASCII/Unicode → 字符：(char)n
-数字 0-9 → 字符 '0'-'9'，最常用：(char)(n + '0')</v>
-      </c>
-      <c r="B4" t="str">
-        <v>int变成char，必须强转 (char)</v>
-      </c>
-      <c r="C4" t="str" xml:space="preserve">
-        <v xml:space="preserve">数字 0-9 → 字符 '0'-'9'，最常用：(char)(n + '0')
-如果你有整数值（0-127）想得到对应字符：
-int n = 65;
-char c = (char) n;
-System.out.println(c);  // 输出 'A'
-ASCII/Unicode → 字符：(char)n</v>
-      </c>
-      <c r="D4" t="str" xml:space="preserve">
-        <v xml:space="preserve">int n = 5;
-char c = (char) (n + '0');
-System.out.println(c);  // 输出 '5'</v>
-      </c>
-    </row>
-    <row r="5" xml:space="preserve">
-      <c r="A5" t="str">
-        <v>res = res * 10 + (c - '0');</v>
-      </c>
-      <c r="B5" t="str">
-        <v>构造数字回文 / 字符串编码：</v>
-      </c>
-      <c r="C5" t="str">
-        <v/>
-      </c>
-      <c r="D5" t="str" xml:space="preserve">
-        <v xml:space="preserve">String s = "123";
-int res = 0;
-for(char c : s.toCharArray()){
-    res = res * 10 + (c - '0');
-}//把字符数字拼接到整数末尾</v>
-      </c>
-    </row>
-    <row r="6" xml:space="preserve">
-      <c r="A6" t="str">
-        <v>(char)('A' + n - 1)</v>
-      </c>
-      <c r="B6" t="str">
-        <v>数字映射字母</v>
-      </c>
-      <c r="C6" t="str">
-        <v>n=1 → 'A' + 0 → 'A'</v>
-      </c>
-      <c r="D6" t="str" xml:space="preserve">
-        <v xml:space="preserve">for (int n = 1; n &lt;= 26; n++) {
-    char letter = (char) ('A' + n - 1);
-    System.out.print(letter + " "); 
-}//A B C D E F G H I J K L M N O P Q R S T U V W X Y Z</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>(char)('A' + (n-1)%26)</v>
-      </c>
-      <c r="B7" t="str">
-        <v>循环映射字母</v>
-      </c>
-      <c r="C7" t="str">
-        <v>n&gt;26 循环映射 A-Z</v>
-      </c>
-    </row>
-    <row r="8" xml:space="preserve">
-      <c r="A8" t="str">
-        <v>int index = c - 'a';</v>
-      </c>
-      <c r="B8" t="str">
-        <v>字母转下标</v>
-      </c>
-      <c r="C8" t="str">
-        <v/>
-      </c>
-      <c r="D8" t="str" xml:space="preserve">
-        <v xml:space="preserve">char c = 'c';
-int index = c - 'a';
-System.out.println(index);</v>
-      </c>
-    </row>
-    <row r="9" xml:space="preserve">
-      <c r="A9" t="str">
-        <v>(char)(i + 'a');</v>
-      </c>
-      <c r="B9" t="str">
-        <v>把索引下标变回字母</v>
-      </c>
-      <c r="C9" t="str">
-        <v/>
-      </c>
-      <c r="D9" t="str" xml:space="preserve">
-        <v xml:space="preserve">"int i = 2; // index是2
-char letter = (char)(i + 'a');"</v>
-      </c>
-    </row>
-    <row r="10" xml:space="preserve">
-      <c r="A10" t="str">
-        <v>Character.isLetterOrDigit('a')</v>
-      </c>
-      <c r="B10" t="str">
-        <v>判断 c 是否是 字母或数字</v>
-      </c>
-      <c r="C10" t="str">
-        <v/>
-      </c>
-      <c r="D10" t="str" xml:space="preserve">
-        <v xml:space="preserve">"Character.isLetterOrDigit('a')  // true
-Character.isLetterOrDigit('7')  // true
-Character.isLetterOrDigit('%')  // false
-Character.isLetterOrDigit(' ')  // false"</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Character.isDigit(c)</v>
-      </c>
-      <c r="B11" t="str">
-        <v>判断是否是数字字符</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>Character.isLetter</v>
-      </c>
-      <c r="B12" t="str">
-        <v>判断是否是字母</v>
-      </c>
-    </row>
-    <row r="13" xml:space="preserve">
-      <c r="A13" t="str">
-        <v>Character.isWhitespace()</v>
-      </c>
-      <c r="B13" t="str" xml:space="preserve">
-        <v xml:space="preserve">判断空白字符，去空格
-字符串清洗</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>Character.isUpperCase()</v>
-      </c>
-      <c r="B14" t="str">
-        <v>是否是大写</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>Character.toLowerCase(c);</v>
-      </c>
-      <c r="B15" t="str">
-        <v>变成小写</v>
-      </c>
-    </row>
-    <row r="16" xml:space="preserve">
-      <c r="A16" t="str">
-        <v>"aeiouAEIOU".indexOf(c) &gt;= 0</v>
-      </c>
-      <c r="B16" t="str">
-        <v>c 是否是 元音字母 (vowel)</v>
-      </c>
-      <c r="C16" t="str" xml:space="preserve">
-        <v xml:space="preserve">a e i o u A E I O U
-0 1 2 3 4 …</v>
-      </c>
-      <c r="D16" t="str" xml:space="preserve">
-        <v xml:space="preserve">if ("aeiouAEIOU".indexOf(c) &gt;= 0) {
-    System.out.println("是元音");
-}</v>
-      </c>
-    </row>
-    <row r="17" xml:space="preserve">
-      <c r="A17" t="str" xml:space="preserve">
-        <v xml:space="preserve">for(char c : s.toCharArray()){
-    freq[c - 'a']++;
-}</v>
-      </c>
-      <c r="B17" t="str">
-        <v>创建一个 26个位置的数组统计字母频率</v>
-      </c>
-      <c r="C17" t="str">
-        <v>[0,0,0,0,0....]数组初始值：'b' - 'a' = 1,所以b就等于1这个下标</v>
-      </c>
-      <c r="D17" t="str" xml:space="preserve">
-        <v xml:space="preserve">String s = "banana";
-int[] freq = new int[26];
-for(char c : s.toCharArray()){
-    freq[c - 'a']++;
-}</v>
-      </c>
-    </row>
-    <row r="18" xml:space="preserve">
-      <c r="A18" t="str" xml:space="preserve">
-        <v xml:space="preserve">char c = 'a';
-String s = Character.toString(c);</v>
-      </c>
-      <c r="B18" t="str">
-        <v>char变成string</v>
-      </c>
-      <c r="C18" t="str">
-        <v>new string其实也是建了新对象，每次string都会建新对象</v>
-      </c>
-    </row>
-    <row r="19" xml:space="preserve">
-      <c r="A19" t="str" xml:space="preserve">
-        <v xml:space="preserve">char[] arr = {'h','e','l','l','o'};
-String s = new String(arr); //"hello"</v>
-      </c>
-      <c r="B19" t="str">
-        <v>char[] → String</v>
-      </c>
-      <c r="C19" t="str">
-        <v/>
-      </c>
-      <c r="D19" t="str" xml:space="preserve">
-        <v xml:space="preserve">"方法一 char[] arr = {'h','e','l','l','o'};
-String s = new String(arr);
-System.out.println(s); // hello""
-方法二 char[] arr = {'h','e','l','l','o'};
-String s = String.valueOf(arr);
-System.out.println(s); // hello"</v>
-      </c>
-    </row>
-    <row r="20" xml:space="preserve">
-      <c r="A20" t="str" xml:space="preserve">
-        <v xml:space="preserve">String s = "hello";
-char[] arr = s.toCharArray();</v>
-      </c>
-      <c r="B20" t="str">
-        <v>string-&gt;char[].会创建数组</v>
-      </c>
-      <c r="C20" t="str">
-        <v>使用 charAt()（不创建数组）</v>
-      </c>
-    </row>
-    <row r="21" xml:space="preserve">
-      <c r="A21" t="str">
-        <v>比较单个字符chr == 'c'</v>
-      </c>
-      <c r="B21" t="str">
-        <v>char 比较要用 ==,string比较用equals</v>
-      </c>
-      <c r="C21" t="str">
-        <v/>
-      </c>
-      <c r="D21" t="str" xml:space="preserve">
-        <v xml:space="preserve">if(c == 'A') {
-    countA++;
-} else if(c == 'L') {
-    countL++;
-}</v>
-      </c>
-    </row>
-    <row r="22" xml:space="preserve">
-      <c r="A22" t="str" xml:space="preserve">
-        <v xml:space="preserve">String s = "abc1";
-boolean allValid = s.chars()
-    .allMatch(c -&gt; Character.isLetterOrDigit(c));
-System.out.println(allValid); // true</v>
-      </c>
-      <c r="B22" t="str">
-        <v>逐个判断每个char是不是数字或字母</v>
-      </c>
-    </row>
-    <row r="23" xml:space="preserve">
-      <c r="A23" t="str" xml:space="preserve">
-        <v xml:space="preserve">char[] arr = {'a','b'};
-System.out.println(arr);因为 println 对 char[] 做了特殊处理。</v>
-      </c>
-    </row>
-  </sheetData>
+  <dimension ref="A1"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D21"/>
+  <sheetData>
+    <row r="1" xml:space="preserve">
+      <c r="A1" t="str" xml:space="preserve">
+        <v xml:space="preserve">char 本质是一个整数（Unicode 编码）_x000d_
+运算时会自动提升为 int（类型提升）_x000d_
+小于 int 的类型（byte / short / char）参与运算 → 自动转成 int_x000d_
+char 比较按 Unicode：'a' &gt; 'A'  // true_x000d_
+_x000d_
+char a = 'A'; // 65_x000d_
+char b = 'B'; // 66_x000d_
+_x000d_
+int result = a + b;</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>方法</v>
+      </c>
+      <c r="B2" t="str">
+        <v>功能</v>
+      </c>
+      <c r="C2" t="str">
+        <v>备注</v>
+      </c>
+      <c r="D2" t="str">
+        <v>例子</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>int n = c - '0'</v>
+      </c>
+      <c r="B3" t="str">
+        <v>char变成int</v>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v>char c = '7';int n = c - '0';   // 7</v>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str" xml:space="preserve">
+        <v xml:space="preserve">char c = (char) (n + '0');_x000d_
+ASCII/Unicode → 字符：(char)n_x000d_
+数字 0-9 → 字符 '0'-'9'，最常用：(char)(n + '0')</v>
+      </c>
+      <c r="B4" t="str">
+        <v>int变成char，必须强转 (char)</v>
+      </c>
+      <c r="C4" t="str" xml:space="preserve">
+        <v xml:space="preserve">数字 0-9 → 字符 '0'-'9'，最常用：(char)(n + '0')_x000d_
+如果你有整数值（0-127）想得到对应字符：_x000d_
+int n = 65;_x000d_
+char c = (char) n;_x000d_
+System.out.println(c);  // 输出 'A'_x000d_
+ASCII/Unicode → 字符：(char)n</v>
+      </c>
+      <c r="D4" t="str" xml:space="preserve">
+        <v xml:space="preserve">int n = 5;_x000d_
+char c = (char) (n + '0');_x000d_
+System.out.println(c);  // 输出 '5'</v>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
+      <c r="A5" t="str">
+        <v>res = res * 10 + (c - '0');</v>
+      </c>
+      <c r="B5" t="str">
+        <v>构造数字回文 / 字符串编码：</v>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str" xml:space="preserve">
+        <v xml:space="preserve">String s = "123";_x000d_
+int res = 0;_x000d_
+_x000d_
+for(char c : s.toCharArray()){_x000d_
+    res = res * 10 + (c - '0');_x000d_
+}//把字符数字拼接到整数末尾</v>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6" t="str">
+        <v>(char)('A' + n - 1)</v>
+      </c>
+      <c r="B6" t="str">
+        <v>数字映射字母</v>
+      </c>
+      <c r="C6" t="str">
+        <v>n=1 → 'A' + 0 → 'A'</v>
+      </c>
+      <c r="D6" t="str" xml:space="preserve">
+        <v xml:space="preserve">for (int n = 1; n &lt;= 26; n++) {_x000d_
+    char letter = (char) ('A' + n - 1);_x000d_
+    System.out.print(letter + " "); _x000d_
+}//A B C D E F G H I J K L M N O P Q R S T U V W X Y Z</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>(char)('A' + (n-1)%26)</v>
+      </c>
+      <c r="B7" t="str">
+        <v>循环映射字母</v>
+      </c>
+      <c r="C7" t="str">
+        <v>n&gt;26 循环映射 A-Z</v>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
+      <c r="A8" t="str">
+        <v>int index = c - 'a';</v>
+      </c>
+      <c r="B8" t="str">
+        <v>字母转下标</v>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+      <c r="D8" t="str" xml:space="preserve">
+        <v xml:space="preserve">char c = 'c';_x000d_
+_x000d_
+int index = c - 'a';_x000d_
+_x000d_
+System.out.println(index);</v>
+      </c>
+    </row>
+    <row r="9" xml:space="preserve">
+      <c r="A9" t="str">
+        <v>(char)(i + 'a');</v>
+      </c>
+      <c r="B9" t="str">
+        <v>把索引下标变回字母</v>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str" xml:space="preserve">
+        <v xml:space="preserve">"int i = 2; // index是2_x000d_
+char letter = (char)(i + 'a');"</v>
+      </c>
+    </row>
+    <row r="10" xml:space="preserve">
+      <c r="A10" t="str">
+        <v>Character.isLetterOrDigit('a')</v>
+      </c>
+      <c r="B10" t="str">
+        <v>判断 c 是否是 字母或数字</v>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+      <c r="D10" t="str" xml:space="preserve">
+        <v xml:space="preserve">"Character.isLetterOrDigit('a')  // true_x000d_
+Character.isLetterOrDigit('7')  // true_x000d_
+Character.isLetterOrDigit('%')  // false_x000d_
+Character.isLetterOrDigit(' ')  // false"</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Character.isDigit(c)</v>
+      </c>
+      <c r="B11" t="str">
+        <v>判断是否是数字字符</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Character.isLetter</v>
+      </c>
+      <c r="B12" t="str">
+        <v>判断是否是字母</v>
+      </c>
+    </row>
+    <row r="13" xml:space="preserve">
+      <c r="A13" t="str">
+        <v>Character.isWhitespace()</v>
+      </c>
+      <c r="B13" t="str" xml:space="preserve">
+        <v xml:space="preserve">判断空白字符，去空格_x000d_
+字符串清洗</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Character.isUpperCase()</v>
+      </c>
+      <c r="B14" t="str">
+        <v>是否是大写</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Character.toLowerCase(c);</v>
+      </c>
+      <c r="B15" t="str">
+        <v>变成小写</v>
+      </c>
+    </row>
+    <row r="16" xml:space="preserve">
+      <c r="A16" t="str">
+        <v>"aeiouAEIOU".indexOf(c) &gt;= 0</v>
+      </c>
+      <c r="B16" t="str">
+        <v>c 是否是 元音字母 (vowel)</v>
+      </c>
+      <c r="C16" t="str" xml:space="preserve">
+        <v xml:space="preserve">a e i o u A E I O U_x000d_
+0 1 2 3 4 …</v>
+      </c>
+      <c r="D16" t="str" xml:space="preserve">
+        <v xml:space="preserve">if ("aeiouAEIOU".indexOf(c) &gt;= 0) {_x000d_
+    System.out.println("是元音");_x000d_
+}</v>
+      </c>
+    </row>
+    <row r="17" xml:space="preserve">
+      <c r="A17" t="str" xml:space="preserve">
+        <v xml:space="preserve">for(char c : s.toCharArray()){_x000d_
+    freq[c - 'a']++;_x000d_
+}</v>
+      </c>
+      <c r="B17" t="str">
+        <v>创建一个 26个位置的数组统计字母频率</v>
+      </c>
+      <c r="C17" t="str">
+        <v>[0,0,0,0,0....]数组初始值：'b' - 'a' = 1,所以b就等于1这个下标</v>
+      </c>
+      <c r="D17" t="str" xml:space="preserve">
+        <v xml:space="preserve">String s = "banana";_x000d_
+_x000d_
+int[] freq = new int[26];_x000d_
+_x000d_
+for(char c : s.toCharArray()){_x000d_
+    freq[c - 'a']++;_x000d_
+}</v>
+      </c>
+    </row>
+    <row r="18" xml:space="preserve">
+      <c r="A18" t="str" xml:space="preserve">
+        <v xml:space="preserve">char c = 'a';_x000d_
+String s = Character.toString(c);</v>
+      </c>
+      <c r="B18" t="str">
+        <v>char变成string</v>
+      </c>
+      <c r="C18" t="str">
+        <v>new string其实也是建了新对象，每次string都会建新对象</v>
+      </c>
+    </row>
+    <row r="19" xml:space="preserve">
+      <c r="A19" t="str" xml:space="preserve">
+        <v xml:space="preserve">char[] arr = {'h','e','l','l','o'};_x000d_
+String s = new String(arr); //"hello"</v>
+      </c>
+      <c r="B19" t="str">
+        <v>char[] → String</v>
+      </c>
+      <c r="C19" t="str">
+        <v/>
+      </c>
+      <c r="D19" t="str" xml:space="preserve">
+        <v xml:space="preserve">"方法一 char[] arr = {'h','e','l','l','o'};_x000d_
+String s = new String(arr);_x000d_
+_x000d_
+System.out.println(s); // hello""_x000d_
+方法二 char[] arr = {'h','e','l','l','o'};_x000d_
+String s = String.valueOf(arr);_x000d_
+_x000d_
+System.out.println(s); // hello"</v>
+      </c>
+    </row>
+    <row r="20" xml:space="preserve">
+      <c r="A20" t="str" xml:space="preserve">
+        <v xml:space="preserve">String s = "hello";_x000d_
+char[] arr = s.toCharArray();</v>
+      </c>
+      <c r="B20" t="str">
+        <v>string-&gt;char[].会创建数组</v>
+      </c>
+      <c r="C20" t="str">
+        <v>使用 charAt()（不创建数组）</v>
+      </c>
+    </row>
+    <row r="21" xml:space="preserve">
+      <c r="A21" t="str" xml:space="preserve">
+        <v xml:space="preserve">char[] arr = {'a','b'};_x000d_
+System.out.println(arr);因为 println 对 char[] 做了特殊处理。</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D21"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D12"/>
   <sheetData>
     <row r="1">
@@ -3507,7 +3933,7 @@
         <v>String转数字,String → int</v>
       </c>
       <c r="C2" t="str" xml:space="preserve">
-        <v xml:space="preserve">parseInt 返回基本类型，
+        <v xml:space="preserve">parseInt 返回基本类型，_x000d_
 valueOf 返回对象。</v>
       </c>
       <c r="D2" t="str">
@@ -3525,14 +3951,14 @@
         <v>返回的是 对象 Integer。</v>
       </c>
       <c r="D3" t="str" xml:space="preserve">
-        <v xml:space="preserve">String s = "123";
+        <v xml:space="preserve">String s = "123";_x000d_
 Integer n = Integer.valueOf(s);</v>
       </c>
     </row>
     <row r="4" xml:space="preserve">
       <c r="A4" t="str" xml:space="preserve">
-        <v xml:space="preserve">Java 的 int 范围是：
-Integer.MAX_VALUE =  2147483647
+        <v xml:space="preserve">Java 的 int 范围是：_x000d_
+Integer.MAX_VALUE =  2147483647_x000d_
 Integer.MIN_VALUE = -2147483648</v>
       </c>
       <c r="B4" t="str">
@@ -3542,19 +3968,19 @@
         <v>[-2^31 , 2^31 - 1]</v>
       </c>
       <c r="D4" t="str" xml:space="preserve">
-        <v xml:space="preserve">MAX_VALUE / 10 作为临界值，
-result &gt; MAX_VALUE / 10 → 下一步一定溢出，
-如果 result == MAX_VALUE / 10：
-	•	digit &gt; 7 → 溢出
+        <v xml:space="preserve">MAX_VALUE / 10 作为临界值，_x000d_
+result &gt; MAX_VALUE / 10 → 下一步一定溢出，_x000d_
+如果 result == MAX_VALUE / 10：_x000d_
+	•	digit &gt; 7 → 溢出_x000d_
 	•	digit ≤ 7 → 安全。为什么是 7？因为 MAX_VALUE 的最后一位是 7（2147483647）</v>
       </c>
     </row>
     <row r="5" xml:space="preserve">
       <c r="A5" t="str" xml:space="preserve">
-        <v xml:space="preserve">if (
-    (result &gt; Integer.MAX_VALUE / 10) ||
-    (result == Integer.MAX_VALUE / 10 &amp;&amp;
-        digit &gt; Integer.MAX_VALUE % 10)
+        <v xml:space="preserve">if (_x000d_
+    (result &gt; Integer.MAX_VALUE / 10) ||_x000d_
+    (result == Integer.MAX_VALUE / 10 &amp;&amp;_x000d_
+        digit &gt; Integer.MAX_VALUE % 10)_x000d_
 )</v>
       </c>
       <c r="B5" t="str">
@@ -3564,17 +3990,17 @@
         <v/>
       </c>
       <c r="D5" t="str" xml:space="preserve">
-        <v xml:space="preserve">String s = "2147483647"; // 正好是 MAX_VALUE
-int result = 0;
-for(char c : s.toCharArray()){
-    int digit = c - '0';
-    // 检查溢出
-    if(result &gt; Integer.MAX_VALUE / 10 || (result == Integer.MAX_VALUE / 10 &amp;&amp; digit &gt; 7)){
-        System.out.println("溢出");
-        break;
-    }
-    result = result * 10 + digit;
-}
+        <v xml:space="preserve">String s = "2147483647"; // 正好是 MAX_VALUE_x000d_
+int result = 0;_x000d_
+for(char c : s.toCharArray()){_x000d_
+    int digit = c - '0';_x000d_
+    // 检查溢出_x000d_
+    if(result &gt; Integer.MAX_VALUE / 10 || (result == Integer.MAX_VALUE / 10 &amp;&amp; digit &gt; 7)){_x000d_
+        System.out.println("溢出");_x000d_
+        break;_x000d_
+    }_x000d_
+    result = result * 10 + digit;_x000d_
+}_x000d_
 System.out.println(result);</v>
       </c>
     </row>
@@ -3665,13 +4091,14 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:D12"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:A16"/>
   <sheetData>
@@ -3682,11 +4109,11 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str" xml:space="preserve">
-        <v xml:space="preserve">在 Java 8 引入的 Stream API 中，流（Stream）是用来操作数据集合的。
-	•	普通对象流（Object Stream） → Stream&lt;T&gt;
-	•	元素是对象，比如 Stream&lt;String&gt; 或 Stream&lt;Integer&gt;
-	•	基本类型流（Primitive Stream） → IntStream, LongStream, DoubleStream，不能直接用泛型
-	•	元素是 Java 的基本类型（int、long、double）
+        <v xml:space="preserve">在 Java 8 引入的 Stream API 中，流（Stream）是用来操作数据集合的。_x000d_
+	•	普通对象流（Object Stream） → Stream&lt;T&gt;_x000d_
+	•	元素是对象，比如 Stream&lt;String&gt; 或 Stream&lt;Integer&gt;_x000d_
+	•	基本类型流（Primitive Stream） → IntStream, LongStream, DoubleStream，不能直接用泛型_x000d_
+	•	元素是 Java 的基本类型（int、long、double）_x000d_
 	•	目的是 性能优化，避免频繁装箱/拆箱</v>
       </c>
     </row>
@@ -3722,7 +4149,7 @@
     </row>
     <row r="9" xml:space="preserve">
       <c r="A9" t="str" xml:space="preserve">
-        <v xml:space="preserve">👉 a 存的是数字
+        <v xml:space="preserve">👉 a 存的是数字_x000d_
 👉 b 存的是对象</v>
       </c>
     </row>
@@ -3733,9 +4160,10 @@
     </row>
     <row r="11" xml:space="preserve">
       <c r="A11" t="str" xml:space="preserve">
-        <v xml:space="preserve">Integer a = Integer.valueOf(10);//返回：对象 Integer
-Integer b = Integer.valueOf("123");
-System.out.println(a);  // 10
+        <v xml:space="preserve">Integer a = Integer.valueOf(10);//返回：对象 Integer_x000d_
+Integer b = Integer.valueOf("123");_x000d_
+_x000d_
+System.out.println(a);  // 10_x000d_
 System.out.println(b);  // 123</v>
       </c>
     </row>
@@ -3746,10 +4174,10 @@
     </row>
     <row r="13" xml:space="preserve">
       <c r="A13" t="str" xml:space="preserve">
-        <v xml:space="preserve">1.	统计频率：getOrDefault + put 或 merge
-	2.	查找 complement / 组合：containsKey
-	3.	分组：computeIfAbsent + List/Set
-	4.	滑动窗口 + HashMap：存字符索引
+        <v xml:space="preserve">1.	统计频率：getOrDefault + put 或 merge_x000d_
+	2.	查找 complement / 组合：containsKey_x000d_
+	3.	分组：computeIfAbsent + List/Set_x000d_
+	4.	滑动窗口 + HashMap：存字符索引_x000d_
 	5.	记录最新位置 / 索引：put 直接覆盖</v>
       </c>
     </row>
@@ -3769,13 +4197,14 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:A16"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D12"/>
   <sheetData>
@@ -3804,13 +4233,15 @@
         <v/>
       </c>
       <c r="D2" t="str" xml:space="preserve">
-        <v xml:space="preserve">Set&lt;Integer&gt; set1 = new HashSet&lt;&gt;();
-set1.add(1);
-set1.add(2);
-Set&lt;Integer&gt; set2 = new HashSet&lt;&gt;();
-set2.add(2);
-set2.add(3);
-set1.addAll(set2);
+        <v xml:space="preserve">Set&lt;Integer&gt; set1 = new HashSet&lt;&gt;();_x000d_
+set1.add(1);_x000d_
+set1.add(2);_x000d_
+_x000d_
+Set&lt;Integer&gt; set2 = new HashSet&lt;&gt;();_x000d_
+set2.add(2);_x000d_
+set2.add(3);_x000d_
+_x000d_
+set1.addAll(set2);_x000d_
 System.out.println(set1);//[1, 2, 3]</v>
       </c>
     </row>
@@ -3825,9 +4256,11 @@
         <v/>
       </c>
       <c r="D3" t="str" xml:space="preserve">
-        <v xml:space="preserve">Set&lt;Integer&gt; set1 = new HashSet&lt;&gt;(Set.of(1, 2, 3));
-Set&lt;Integer&gt; set2 = new HashSet&lt;&gt;(Set.of(2, 3, 4));
-set1.retainAll(set2);  // 只保留同时在 set1 和 set2 中的元素
+        <v xml:space="preserve">Set&lt;Integer&gt; set1 = new HashSet&lt;&gt;(Set.of(1, 2, 3));_x000d_
+Set&lt;Integer&gt; set2 = new HashSet&lt;&gt;(Set.of(2, 3, 4));_x000d_
+_x000d_
+set1.retainAll(set2);  // 只保留同时在 set1 和 set2 中的元素_x000d_
+_x000d_
 System.out.println(set1);//[2, 3]</v>
       </c>
     </row>
@@ -3836,17 +4269,19 @@
         <v>set.removeAll(set2);</v>
       </c>
       <c r="B4" t="str" xml:space="preserve">
-        <v xml:space="preserve">删除集合中同时存在于另一个集合的元素，差集，[1,2,3] - [2,3,4]
+        <v xml:space="preserve">删除集合中同时存在于另一个集合的元素，差集，[1,2,3] - [2,3,4]_x000d_
 [1]</v>
       </c>
       <c r="C4" t="str" xml:space="preserve">
-        <v xml:space="preserve">set1.removeAll(set2)
+        <v xml:space="preserve">set1.removeAll(set2)_x000d_
 = 删除 set1 中所有也在 set2 的元素</v>
       </c>
       <c r="D4" t="str" xml:space="preserve">
-        <v xml:space="preserve">Set&lt;Integer&gt; set1 = new HashSet&lt;&gt;(Set.of(1, 2, 3, 4));
-Set&lt;Integer&gt; set2 = new HashSet&lt;&gt;(Set.of(2, 3, 5));
-set1.removeAll(set2);  // 删除 set1 中所有在 set2 中的元素
+        <v xml:space="preserve">Set&lt;Integer&gt; set1 = new HashSet&lt;&gt;(Set.of(1, 2, 3, 4));_x000d_
+Set&lt;Integer&gt; set2 = new HashSet&lt;&gt;(Set.of(2, 3, 5));_x000d_
+_x000d_
+set1.removeAll(set2);  // 删除 set1 中所有在 set2 中的元素_x000d_
+_x000d_
 System.out.println(set1);//[1, 4]</v>
       </c>
     </row>
@@ -3942,14 +4377,15 @@
         <v>是否包含元素</v>
       </c>
       <c r="C11" t="str" xml:space="preserve">
-        <v xml:space="preserve">返回 true → 新增成功，
+        <v xml:space="preserve">返回 true → 新增成功，_x000d_
 重复元素返回 false</v>
       </c>
       <c r="D11" t="str" xml:space="preserve">
-        <v xml:space="preserve">Set&lt;String&gt; set = new HashSet&lt;&gt;();
-set.add("apple");
-set.add("banana");
-set.add("orange");
+        <v xml:space="preserve">Set&lt;String&gt; set = new HashSet&lt;&gt;();_x000d_
+set.add("apple");_x000d_
+set.add("banana");_x000d_
+set.add("orange");_x000d_
+_x000d_
 System.out.println(set.contains("banana"));  // true</v>
       </c>
     </row>
@@ -3968,289 +4404,9 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:D12"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D21"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>方法</v>
-      </c>
-      <c r="B1" t="str">
-        <v>功能</v>
-      </c>
-      <c r="C1" t="str">
-        <v>备注</v>
-      </c>
-      <c r="D1" t="str">
-        <v>例子</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Map&lt;String, Integer&gt; map = new HashMap&lt;&gt;();</v>
-      </c>
-      <c r="B2" t="str">
-        <v>创建一个空 HashMap</v>
-      </c>
-    </row>
-    <row r="3" xml:space="preserve">
-      <c r="A3" t="str" xml:space="preserve">
-        <v xml:space="preserve">map.put("apple", 3); // 添加 key=apple, value=3
-map.put("banana", 5); // 添加
-map.put("apple", 10); // 更新 key=apple 的值为10</v>
-      </c>
-      <c r="B3" t="str">
-        <v>添加 / 更新元素</v>
-      </c>
-    </row>
-    <row r="4" xml:space="preserve">
-      <c r="A4" t="str">
-        <v>map.put(key, map.getOrDefault(key, 0) + 1);</v>
-      </c>
-      <c r="B4" t="str">
-        <v>统计频率</v>
-      </c>
-      <c r="C4" t="str" xml:space="preserve">
-        <v xml:space="preserve">如果 key 已存在 → value +1
-如果 key 不存在 → 默认 0 +1 → 放入 1</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>map.getOrDefault("orange", 0);</v>
-      </c>
-      <c r="B5" t="str">
-        <v>统计出现次数，获取元素</v>
-      </c>
-      <c r="C5" t="str">
-        <v>int val2 = map.getOrDefault("orange", 0); // 不存在返回0</v>
-      </c>
-    </row>
-    <row r="6" xml:space="preserve">
-      <c r="A6" t="str" xml:space="preserve">
-        <v xml:space="preserve">map.containsKey("apple"); // true
-map.containsValue(10);    // true</v>
-      </c>
-      <c r="B6" t="str">
-        <v>判断 key / value</v>
-      </c>
-      <c r="C6" t="str" xml:space="preserve">
-        <v xml:space="preserve">map.containsKey("apple"); // true
-map.containsValue(10);    // true</v>
-      </c>
-    </row>
-    <row r="7" xml:space="preserve">
-      <c r="A7" t="str" xml:space="preserve">
-        <v xml:space="preserve">map.remove("banana");       // 删除 key=banana
-map.remove("apple", 10);    // 删除 key=apple 且 value=10 的条目</v>
-      </c>
-      <c r="B7" t="str">
-        <v>删除元素</v>
-      </c>
-    </row>
-    <row r="8" xml:space="preserve">
-      <c r="A8" t="str" xml:space="preserve">
-        <v xml:space="preserve">for (String key : map.keySet()) {
-    System.out.println(key + " -&gt; " + map.get(key));
-}</v>
-      </c>
-      <c r="B8" t="str">
-        <v>遍历 key</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>for (Integer value : map.values()) {System.out.println(value);}</v>
-      </c>
-      <c r="B9" t="str">
-        <v>遍历value</v>
-      </c>
-    </row>
-    <row r="10" xml:space="preserve">
-      <c r="A10" t="str" xml:space="preserve">
-        <v xml:space="preserve">for (Map.Entry&lt;String, Integer&gt; entry : map.entrySet()) {
-    System.out.println(entry.getKey() + " -&gt; " + entry.getValue());
-}</v>
-      </c>
-      <c r="B10" t="str">
-        <v>遍历Entry</v>
-      </c>
-    </row>
-    <row r="11" xml:space="preserve">
-      <c r="A11" t="str" xml:space="preserve">
-        <v xml:space="preserve">map.computeIfAbsent(key, k -&gt; value);
-如果没有 key，就创建新的 ArrayList
-            indexMap.computeIfAbsent(c, k -&gt; new ArrayList&lt;&gt;()).add(i);</v>
-      </c>
-      <c r="B11" t="str" xml:space="preserve">
-        <v xml:space="preserve">分组：computeIfAbsent
-map.computeIfAbsent("A", k -&gt; new ArrayList&lt;&gt;()).add(1);</v>
-      </c>
-      <c r="C11" t="str" xml:space="preserve">
-        <v xml:space="preserve">当 value 是 List / Set / Map 时初始化：
-map.computeIfAbsent(key, k -&gt; new ArrayList&lt;&gt;()).add(value);</v>
-      </c>
-      <c r="D11" t="str" xml:space="preserve">
-        <v xml:space="preserve">Map&lt;Character, List&lt;String&gt;&gt; map = new HashMap&lt;&gt;();
-String[] words = {"apple","ant","banana","boat"};
-for(String w : words){
-    char c = w.charAt(0);
-    map.computeIfAbsent(c, k -&gt; new ArrayList&lt;&gt;()).add(w);
-}
-System.out.println(map);
-------------------------------------
-Map&lt;String, Integer&gt; count = new HashMap&lt;&gt;();
-String[] words = {"apple", "banana", "apple", "orange", "banana"};
-for (String word : words) {
-    count.computeIfAbsent(word, k -&gt; 0); // 如果没有 key，word就是关键词 ，值初始化为 0
-    count.put(word, count.get(word) + 1); // 再 +1
-}
-System.out.println(count);</v>
-      </c>
-    </row>
-    <row r="12" xml:space="preserve">
-      <c r="A12" t="str">
-        <v>map.putIfAbsent(key, value);</v>
-      </c>
-      <c r="B12" t="str">
-        <v>putIfAbsent只在不存在时放入，如果 key 已存在 → 不覆盖，初始化默认值</v>
-      </c>
-      <c r="C12" t="str" xml:space="preserve">
-        <v xml:space="preserve">需要你自己创建 value，
-put() 会覆盖旧值。</v>
-      </c>
-      <c r="D12" t="str" xml:space="preserve">
-        <v xml:space="preserve">Map&lt;String, List&lt;Integer&gt;&gt; map = new HashMap&lt;&gt;();
-map.putIfAbsent("A", new ArrayList&lt;&gt;());
-map.get("A").add(1);
-map.putIfAbsent("A", new ArrayList&lt;&gt;());
-map.get("A").add(2);
-System.out.println(map);//{A=[1, 2]}
-------------------------------------------
-Map&lt;String, Integer&gt; map = new HashMap&lt;&gt;();
-map.put("A", 10);
-map.putIfAbsent("A", 20);   // A 已存在，不会覆盖
-map.putIfAbsent("B", 30);   // B 不存在，会添加
-System.out.println(map);//{A=10, B=30} 因为A已经有了，所以即使加进去也没用</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>map.replace(key, oldVal, newVal)</v>
-      </c>
-      <c r="B13" t="str">
-        <v>替换指定 key 的值（如果值是 oldVal）</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>map.clear()</v>
-      </c>
-      <c r="B14" t="str">
-        <v>清空整个 Map</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>map.isEmpty()</v>
-      </c>
-      <c r="B15" t="str">
-        <v>判断是否为空</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>map.merge(key, value, BiFunction)</v>
-      </c>
-      <c r="B16" t="str">
-        <v>合并 value，例如累加频率</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>map.forEach((k,v) -&gt; {})</v>
-      </c>
-      <c r="B17" t="str">
-        <v>Java 8 lambda 遍历</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>map.merge(key, 1, Integer::sum);</v>
-      </c>
-      <c r="B18" t="str">
-        <v>如果没有key，就1，有的话， 就累加sum</v>
-      </c>
-      <c r="C18" t="str">
-        <v>merge（最优雅计数法）计数 &amp; 累加，多用于字符统计，找重复元素</v>
-      </c>
-    </row>
-    <row r="19" xml:space="preserve">
-      <c r="A19" t="str">
-        <v>map.merge(key, 1, Integer::sum);</v>
-      </c>
-      <c r="B19" t="str">
-        <v>字符统计</v>
-      </c>
-      <c r="C19" t="str">
-        <v/>
-      </c>
-      <c r="D19" t="str" xml:space="preserve">
-        <v xml:space="preserve">Map&lt;Character, Integer&gt; count = new HashMap&lt;&gt;();
-for (char c : "banana".toCharArray()) {
-    count.merge(c, 1, Integer::sum);
-}
-System.out.println(count);//{b=1, a=3, n=2}
--------------------------------
-if (map.merge(num, 1, Integer::sum) &gt; 1) {
-    // duplicate
-}</v>
-      </c>
-    </row>
-    <row r="20" xml:space="preserve">
-      <c r="A20" t="str">
-        <v>map.compute(key, (k, v) -&gt; v == null ? 1 : v + 1);</v>
-      </c>
-      <c r="B20" t="str">
-        <v>compute（万能函数），功能和 getOrDefault 类似，但更灵活。	统计频率</v>
-      </c>
-      <c r="C20" t="str" xml:space="preserve">
-        <v xml:space="preserve">如果 key 不存在 → value = 1
-如果 key 已存在 → value + 1</v>
-      </c>
-      <c r="D20" t="str" xml:space="preserve">
-        <v xml:space="preserve">Map&lt;Character, Integer&gt; map = new HashMap&lt;&gt;();
-for(char c : "banana".toCharArray()){
-    map.compute(c, (k, v) -&gt; v == null ? 1 : v + 1);
-}
-System.out.println(map);//{b=1, a=3, n=2}</v>
-      </c>
-    </row>
-    <row r="21" xml:space="preserve">
-      <c r="A21" t="str" xml:space="preserve">
-        <v xml:space="preserve">1.	map.getOrDefault(c, someDefault)
-	2.	map.putIfAbsent(c, nextLetter)</v>
-      </c>
-      <c r="B21" t="str" xml:space="preserve">
-        <v xml:space="preserve">•	如果 c 在 map 中有值，返回值
-•	如果没有，返回 someDefault</v>
-      </c>
-      <c r="C21" t="str" xml:space="preserve">
-        <v xml:space="preserve">putIfAbsent
-•	如果 c 不存在，则放入 nextLetter
-•	如果已经存在，保持原来的映射，这样就天然忽略重复字母，只给第一次出现的字母分配映射。</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D21"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>